<commit_message>
Burn Rate Forecast: color-code % Used cells to match chart zones, clarify 70% Line column
</commit_message>
<xml_diff>
--- a/client/public/examples/cost-and-burn-rate-tracker.xlsx
+++ b/client/public/examples/cost-and-burn-rate-tracker.xlsx
@@ -6823,8 +6823,8 @@
       </c>
       <c r="G14" s="137" t="inlineStr">
         <is>
-          <t>70%
-Line</t>
+          <t>Chart Ref
+Only: 70%</t>
         </is>
       </c>
       <c r="I14" s="117" t="inlineStr">
@@ -7784,6 +7784,50 @@
     </cfRule>
     <cfRule type="expression" priority="12" dxfId="13">
       <formula>B10&lt;0.5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C15:C38">
+    <cfRule type="expression" priority="13" dxfId="11">
+      <formula>C15&gt;=0.7</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="12">
+      <formula>AND(C15&gt;=0.5,C15&lt;0.7)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="13">
+      <formula>C15&lt;0.5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D15:D38">
+    <cfRule type="expression" priority="16" dxfId="11">
+      <formula>D15&gt;=0.7</formula>
+    </cfRule>
+    <cfRule type="expression" priority="17" dxfId="12">
+      <formula>AND(D15&gt;=0.5,D15&lt;0.7)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="18" dxfId="13">
+      <formula>D15&lt;0.5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E15:E38">
+    <cfRule type="expression" priority="19" dxfId="11">
+      <formula>E15&gt;=0.7</formula>
+    </cfRule>
+    <cfRule type="expression" priority="20" dxfId="12">
+      <formula>AND(E15&gt;=0.5,E15&lt;0.7)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="21" dxfId="13">
+      <formula>E15&lt;0.5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F15:F38">
+    <cfRule type="expression" priority="22" dxfId="11">
+      <formula>F15&gt;=0.7</formula>
+    </cfRule>
+    <cfRule type="expression" priority="23" dxfId="12">
+      <formula>AND(F15&gt;=0.5,F15&lt;0.7)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="24" dxfId="13">
+      <formula>F15&lt;0.5</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
FundingMods: add ACRN/SLIN columns, reconcile log vs Projects tab
- Each mod log entry now carries an ACRN and SLIN so funding can be
  tracked down to the actual funding line, not just its CLIN.
- New CLIN Funding Status columns: Mod Log Total $ (sum of this
  log's own entries) vs Funded $ (from Projects, the source of
  truth), with a Match/MISMATCH flag per CLIN and overall — catches
  the case where someone updates one tab without the other.
</commit_message>
<xml_diff>
--- a/client/public/examples/cost-and-burn-rate-tracker.xlsx
+++ b/client/public/examples/cost-and-burn-rate-tracker.xlsx
@@ -28,6 +28,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'ODCs'!$A$4:$F$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Travel'!$A$4:$F$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'M&amp;E'!$A$4:$F$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'FundingMods'!$A$4:$P$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -563,7 +564,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="242">
+  <cellXfs count="232">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1100,49 +1101,13 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="28" fillId="19" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1183,6 +1148,12 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1201,7 +1172,7 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
     <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="17">
     <dxf>
       <fill>
         <patternFill>
@@ -1322,6 +1293,29 @@
           <fgColor rgb="FFDCEEDC"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FF3B6D11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDCEEDC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FF3B6D11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FF9C1C1C"/>
+      </font>
     </dxf>
   </dxfs>
   <colors>
@@ -1912,47 +1906,31 @@
 
 <file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
+  <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <to>
-      <col>0</col>
-      <colOff>247320</colOff>
-      <row>0</row>
-      <rowOff>247320</rowOff>
-    </to>
+    <ext cx="266700" cy="266700"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="3" name="Image 1" descr="Picture"/>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="0"/>
-          <a:ext cx="247320" cy="247320"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
-  </twoCellAnchor>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -7837,666 +7815,825 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
+  <sheetPr>
     <tabColor rgb="FFEF9F27"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <dimension ref="A1:P26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" style="108" min="1" max="1"/>
-    <col width="12" customWidth="1" style="108" min="2" max="2"/>
-    <col width="34" customWidth="1" style="108" min="3" max="3"/>
-    <col width="14" customWidth="1" style="108" min="4" max="4"/>
-    <col width="13" customWidth="1" style="108" min="5" max="9"/>
-    <col width="14" customWidth="1" style="108" min="10" max="14"/>
+    <col width="17" customWidth="1" style="109" min="1" max="1"/>
+    <col width="13" customWidth="1" style="109" min="2" max="2"/>
+    <col width="13" customWidth="1" style="109" min="3" max="3"/>
+    <col width="16" customWidth="1" style="109" min="4" max="4"/>
+    <col width="34" customWidth="1" style="109" min="5" max="5"/>
+    <col width="14" customWidth="1" style="109" min="6" max="6"/>
+    <col width="13" customWidth="1" style="109" min="7" max="7"/>
+    <col width="13" customWidth="1" style="109" min="8" max="8"/>
+    <col width="13" customWidth="1" style="109" min="9" max="9"/>
+    <col width="13" customWidth="1" style="109" min="10" max="10"/>
+    <col width="13" customWidth="1" style="109" min="11" max="11"/>
+    <col width="13" customWidth="1" style="109" min="12" max="12"/>
+    <col width="13" customWidth="1" style="109" min="13" max="13"/>
+    <col width="13" customWidth="1" style="109" min="14" max="14"/>
+    <col width="13" customWidth="1" style="109" min="15" max="15"/>
+    <col width="13" customWidth="1" style="109" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="21.75" customHeight="1" s="109">
-      <c r="B1" s="141" t="inlineStr">
+      <c r="B1" s="121" t="inlineStr">
         <is>
           <t>Funding Modification Log</t>
         </is>
       </c>
-      <c r="N1" s="142" t="inlineStr">
+      <c r="P1" s="122" t="inlineStr">
         <is>
           <t>Acqlerate  ·  acqlerate.com</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1" s="109">
-      <c r="A3" s="164" t="inlineStr">
-        <is>
-          <t>HISTORICAL AUDIT LOG — for reference only. This no longer feeds the Dashboard or the CLIN Funding Status table below; those now read live TOA from the Projects tab. Keep logging mods here anyway — it's the paper trail a real contract needs, split across CLIN and (optionally) Project the same way as before.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="33.75" customHeight="1" s="109">
-      <c r="A4" s="151" t="inlineStr">
+    <row r="3" ht="48" customHeight="1" s="109">
+      <c r="A3" s="114" t="inlineStr">
+        <is>
+          <t>HISTORICAL AUDIT LOG — for reference only. This no longer feeds the Dashboard or the CLIN Funding Status table below; those now read live TOA from the Projects tab. Keep logging mods here anyway — it's the paper trail a real contract needs. ACRN and SLIN let you track each mod down to its actual funding line, not just its CLIN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1" s="109">
+      <c r="A4" s="126" t="inlineStr">
         <is>
           <t>Mod #</t>
         </is>
       </c>
-      <c r="B4" s="151" t="inlineStr">
+      <c r="B4" s="126" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C4" s="151" t="inlineStr">
+      <c r="C4" s="126" t="inlineStr">
+        <is>
+          <t>ACRN</t>
+        </is>
+      </c>
+      <c r="D4" s="126" t="inlineStr">
+        <is>
+          <t>SLIN</t>
+        </is>
+      </c>
+      <c r="E4" s="126" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D4" s="210" t="inlineStr">
+      <c r="F4" s="126" t="inlineStr">
         <is>
           <t>Project
 (optional)</t>
         </is>
       </c>
-      <c r="E4" s="151" t="inlineStr">
+      <c r="G4" s="126" t="inlineStr">
         <is>
           <t>Labor CLIN
 $</t>
         </is>
       </c>
-      <c r="F4" s="151" t="inlineStr">
+      <c r="H4" s="126" t="inlineStr">
         <is>
           <t>Travel CLIN
 $</t>
         </is>
       </c>
-      <c r="G4" s="151" t="inlineStr">
+      <c r="I4" s="126" t="inlineStr">
         <is>
           <t>ODC CLIN
 $</t>
         </is>
       </c>
-      <c r="H4" s="151" t="inlineStr">
+      <c r="J4" s="126" t="inlineStr">
         <is>
           <t>M&amp;E CLIN
 $</t>
         </is>
       </c>
-      <c r="I4" s="210" t="inlineStr">
+      <c r="K4" s="126" t="inlineStr">
         <is>
           <t>Mod Total
 $</t>
         </is>
       </c>
-      <c r="J4" s="211" t="inlineStr">
+      <c r="L4" s="126" t="inlineStr">
         <is>
           <t>Cum. Labor
 TOA $</t>
         </is>
       </c>
-      <c r="K4" s="211" t="inlineStr">
+      <c r="M4" s="126" t="inlineStr">
         <is>
           <t>Cum. Travel
 TOA $</t>
         </is>
       </c>
-      <c r="L4" s="211" t="inlineStr">
+      <c r="N4" s="126" t="inlineStr">
         <is>
           <t>Cum. ODC
 TOA $</t>
         </is>
       </c>
-      <c r="M4" s="211" t="inlineStr">
+      <c r="O4" s="126" t="inlineStr">
         <is>
           <t>Cum. M&amp;E
 TOA $</t>
         </is>
       </c>
-      <c r="N4" s="211" t="inlineStr">
+      <c r="P4" s="126" t="inlineStr">
         <is>
           <t>Cum. Total
 TOA $</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="109">
-      <c r="A5" s="165" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="128" t="inlineStr">
         <is>
           <t>P00000 (Award)</t>
         </is>
       </c>
-      <c r="B5" s="169" t="n">
+      <c r="B5" s="202" t="n">
         <v>46023</v>
       </c>
-      <c r="C5" s="165" t="inlineStr">
+      <c r="C5" s="128" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="D5" s="128" t="inlineStr">
+        <is>
+          <t>0001</t>
+        </is>
+      </c>
+      <c r="E5" s="128" t="inlineStr">
         <is>
           <t>Original award — base period</t>
         </is>
       </c>
-      <c r="D5" s="212" t="n"/>
-      <c r="E5" s="166" t="n">
+      <c r="F5" s="128" t="n"/>
+      <c r="G5" s="131" t="n">
         <v>1300000</v>
       </c>
-      <c r="F5" s="166" t="n">
+      <c r="H5" s="131" t="n">
         <v>300000</v>
       </c>
-      <c r="G5" s="166" t="n">
+      <c r="I5" s="131" t="n">
         <v>250000</v>
       </c>
-      <c r="H5" s="166" t="n">
+      <c r="J5" s="131" t="n">
         <v>150000</v>
       </c>
-      <c r="I5" s="213">
-        <f>IF(A5="","",SUM(E5:H5))</f>
-        <v/>
-      </c>
-      <c r="J5" s="154">
-        <f>IF(A5="","",SUM($E$5:E5))</f>
-        <v/>
-      </c>
-      <c r="K5" s="154">
-        <f>IF(A5="","",SUM($F$5:F5))</f>
-        <v/>
-      </c>
-      <c r="L5" s="154">
+      <c r="K5" s="132">
+        <f>IF(A5="","",SUM(G5:J5))</f>
+        <v/>
+      </c>
+      <c r="L5" s="132">
         <f>IF(A5="","",SUM($G$5:G5))</f>
         <v/>
       </c>
-      <c r="M5" s="154">
+      <c r="M5" s="132">
         <f>IF(A5="","",SUM($H$5:H5))</f>
         <v/>
       </c>
-      <c r="N5" s="214">
-        <f>IF(A5="","",J5+K5+L5+M5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="109">
-      <c r="A6" s="172" t="inlineStr">
+      <c r="N5" s="132">
+        <f>IF(A5="","",SUM($I$5:I5))</f>
+        <v/>
+      </c>
+      <c r="O5" s="132">
+        <f>IF(A5="","",SUM($J$5:J5))</f>
+        <v/>
+      </c>
+      <c r="P5" s="132">
+        <f>IF(A5="","",L5+M5+N5+O5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="128" t="inlineStr">
         <is>
           <t>P00001</t>
         </is>
       </c>
-      <c r="B6" s="176" t="n">
+      <c r="B6" s="202" t="n">
         <v>46143</v>
       </c>
-      <c r="C6" s="172" t="inlineStr">
+      <c r="C6" s="128" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="D6" s="128" t="inlineStr">
+        <is>
+          <t>0002</t>
+        </is>
+      </c>
+      <c r="E6" s="128" t="inlineStr">
         <is>
           <t>Incremental funding — added scope</t>
         </is>
       </c>
-      <c r="D6" s="215" t="n"/>
-      <c r="E6" s="173" t="n">
+      <c r="F6" s="128" t="n"/>
+      <c r="G6" s="131" t="n">
         <v>250000</v>
       </c>
-      <c r="F6" s="173" t="n">
+      <c r="H6" s="131" t="n">
         <v>50000</v>
       </c>
-      <c r="G6" s="173" t="n">
+      <c r="I6" s="131" t="n">
         <v>30000</v>
       </c>
-      <c r="H6" s="173" t="n">
+      <c r="J6" s="131" t="n">
         <v>20000</v>
       </c>
-      <c r="I6" s="216">
-        <f>IF(A6="","",SUM(E6:H6))</f>
-        <v/>
-      </c>
-      <c r="J6" s="160">
-        <f>IF(A6="","",SUM($E$5:E6))</f>
-        <v/>
-      </c>
-      <c r="K6" s="160">
-        <f>IF(A6="","",SUM($F$5:F6))</f>
-        <v/>
-      </c>
-      <c r="L6" s="160">
+      <c r="K6" s="132">
+        <f>IF(A6="","",SUM(G6:J6))</f>
+        <v/>
+      </c>
+      <c r="L6" s="132">
         <f>IF(A6="","",SUM($G$5:G6))</f>
         <v/>
       </c>
-      <c r="M6" s="160">
+      <c r="M6" s="132">
         <f>IF(A6="","",SUM($H$5:H6))</f>
         <v/>
       </c>
-      <c r="N6" s="217">
-        <f>IF(A6="","",J6+K6+L6+M6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="109">
-      <c r="A7" s="165" t="n"/>
-      <c r="B7" s="169" t="n"/>
-      <c r="C7" s="165" t="n"/>
-      <c r="D7" s="212" t="n"/>
-      <c r="E7" s="166" t="n"/>
-      <c r="F7" s="166" t="n"/>
-      <c r="G7" s="166" t="n"/>
-      <c r="H7" s="166" t="n"/>
-      <c r="I7" s="213">
-        <f>IF(A7="","",SUM(E7:H7))</f>
-        <v/>
-      </c>
-      <c r="J7" s="154">
-        <f>IF(A7="","",SUM($E$5:E7))</f>
-        <v/>
-      </c>
-      <c r="K7" s="154">
-        <f>IF(A7="","",SUM($F$5:F7))</f>
-        <v/>
-      </c>
-      <c r="L7" s="154">
+      <c r="N6" s="132">
+        <f>IF(A6="","",SUM($I$5:I6))</f>
+        <v/>
+      </c>
+      <c r="O6" s="132">
+        <f>IF(A6="","",SUM($J$5:J6))</f>
+        <v/>
+      </c>
+      <c r="P6" s="132">
+        <f>IF(A6="","",L6+M6+N6+O6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="128" t="n"/>
+      <c r="B7" s="202" t="n"/>
+      <c r="C7" s="128" t="n"/>
+      <c r="D7" s="128" t="n"/>
+      <c r="E7" s="128" t="n"/>
+      <c r="F7" s="128" t="n"/>
+      <c r="G7" s="131" t="n"/>
+      <c r="H7" s="131" t="n"/>
+      <c r="I7" s="131" t="n"/>
+      <c r="J7" s="131" t="n"/>
+      <c r="K7" s="132">
+        <f>IF(A7="","",SUM(G7:J7))</f>
+        <v/>
+      </c>
+      <c r="L7" s="132">
         <f>IF(A7="","",SUM($G$5:G7))</f>
         <v/>
       </c>
-      <c r="M7" s="154">
+      <c r="M7" s="132">
         <f>IF(A7="","",SUM($H$5:H7))</f>
         <v/>
       </c>
-      <c r="N7" s="214">
-        <f>IF(A7="","",J7+K7+L7+M7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="109">
-      <c r="A8" s="172" t="n"/>
-      <c r="B8" s="176" t="n"/>
-      <c r="C8" s="172" t="n"/>
-      <c r="D8" s="215" t="n"/>
-      <c r="E8" s="173" t="n"/>
-      <c r="F8" s="173" t="n"/>
-      <c r="G8" s="173" t="n"/>
-      <c r="H8" s="173" t="n"/>
-      <c r="I8" s="216">
-        <f>IF(A8="","",SUM(E8:H8))</f>
-        <v/>
-      </c>
-      <c r="J8" s="160">
-        <f>IF(A8="","",SUM($E$5:E8))</f>
-        <v/>
-      </c>
-      <c r="K8" s="160">
-        <f>IF(A8="","",SUM($F$5:F8))</f>
-        <v/>
-      </c>
-      <c r="L8" s="160">
+      <c r="N7" s="132">
+        <f>IF(A7="","",SUM($I$5:I7))</f>
+        <v/>
+      </c>
+      <c r="O7" s="132">
+        <f>IF(A7="","",SUM($J$5:J7))</f>
+        <v/>
+      </c>
+      <c r="P7" s="132">
+        <f>IF(A7="","",L7+M7+N7+O7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="128" t="n"/>
+      <c r="B8" s="202" t="n"/>
+      <c r="C8" s="128" t="n"/>
+      <c r="D8" s="128" t="n"/>
+      <c r="E8" s="128" t="n"/>
+      <c r="F8" s="128" t="n"/>
+      <c r="G8" s="131" t="n"/>
+      <c r="H8" s="131" t="n"/>
+      <c r="I8" s="131" t="n"/>
+      <c r="J8" s="131" t="n"/>
+      <c r="K8" s="132">
+        <f>IF(A8="","",SUM(G8:J8))</f>
+        <v/>
+      </c>
+      <c r="L8" s="132">
         <f>IF(A8="","",SUM($G$5:G8))</f>
         <v/>
       </c>
-      <c r="M8" s="160">
+      <c r="M8" s="132">
         <f>IF(A8="","",SUM($H$5:H8))</f>
         <v/>
       </c>
-      <c r="N8" s="217">
-        <f>IF(A8="","",J8+K8+L8+M8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="109">
-      <c r="A9" s="165" t="n"/>
-      <c r="B9" s="169" t="n"/>
-      <c r="C9" s="165" t="n"/>
-      <c r="D9" s="212" t="n"/>
-      <c r="E9" s="166" t="n"/>
-      <c r="F9" s="166" t="n"/>
-      <c r="G9" s="166" t="n"/>
-      <c r="H9" s="166" t="n"/>
-      <c r="I9" s="213">
-        <f>IF(A9="","",SUM(E9:H9))</f>
-        <v/>
-      </c>
-      <c r="J9" s="154">
-        <f>IF(A9="","",SUM($E$5:E9))</f>
-        <v/>
-      </c>
-      <c r="K9" s="154">
-        <f>IF(A9="","",SUM($F$5:F9))</f>
-        <v/>
-      </c>
-      <c r="L9" s="154">
+      <c r="N8" s="132">
+        <f>IF(A8="","",SUM($I$5:I8))</f>
+        <v/>
+      </c>
+      <c r="O8" s="132">
+        <f>IF(A8="","",SUM($J$5:J8))</f>
+        <v/>
+      </c>
+      <c r="P8" s="132">
+        <f>IF(A8="","",L8+M8+N8+O8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="128" t="n"/>
+      <c r="B9" s="202" t="n"/>
+      <c r="C9" s="128" t="n"/>
+      <c r="D9" s="128" t="n"/>
+      <c r="E9" s="128" t="n"/>
+      <c r="F9" s="128" t="n"/>
+      <c r="G9" s="131" t="n"/>
+      <c r="H9" s="131" t="n"/>
+      <c r="I9" s="131" t="n"/>
+      <c r="J9" s="131" t="n"/>
+      <c r="K9" s="132">
+        <f>IF(A9="","",SUM(G9:J9))</f>
+        <v/>
+      </c>
+      <c r="L9" s="132">
         <f>IF(A9="","",SUM($G$5:G9))</f>
         <v/>
       </c>
-      <c r="M9" s="154">
+      <c r="M9" s="132">
         <f>IF(A9="","",SUM($H$5:H9))</f>
         <v/>
       </c>
-      <c r="N9" s="214">
-        <f>IF(A9="","",J9+K9+L9+M9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="109">
-      <c r="A10" s="172" t="n"/>
-      <c r="B10" s="176" t="n"/>
-      <c r="C10" s="172" t="n"/>
-      <c r="D10" s="215" t="n"/>
-      <c r="E10" s="173" t="n"/>
-      <c r="F10" s="173" t="n"/>
-      <c r="G10" s="173" t="n"/>
-      <c r="H10" s="173" t="n"/>
-      <c r="I10" s="216">
-        <f>IF(A10="","",SUM(E10:H10))</f>
-        <v/>
-      </c>
-      <c r="J10" s="160">
-        <f>IF(A10="","",SUM($E$5:E10))</f>
-        <v/>
-      </c>
-      <c r="K10" s="160">
-        <f>IF(A10="","",SUM($F$5:F10))</f>
-        <v/>
-      </c>
-      <c r="L10" s="160">
+      <c r="N9" s="132">
+        <f>IF(A9="","",SUM($I$5:I9))</f>
+        <v/>
+      </c>
+      <c r="O9" s="132">
+        <f>IF(A9="","",SUM($J$5:J9))</f>
+        <v/>
+      </c>
+      <c r="P9" s="132">
+        <f>IF(A9="","",L9+M9+N9+O9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="128" t="n"/>
+      <c r="B10" s="202" t="n"/>
+      <c r="C10" s="128" t="n"/>
+      <c r="D10" s="128" t="n"/>
+      <c r="E10" s="128" t="n"/>
+      <c r="F10" s="128" t="n"/>
+      <c r="G10" s="131" t="n"/>
+      <c r="H10" s="131" t="n"/>
+      <c r="I10" s="131" t="n"/>
+      <c r="J10" s="131" t="n"/>
+      <c r="K10" s="132">
+        <f>IF(A10="","",SUM(G10:J10))</f>
+        <v/>
+      </c>
+      <c r="L10" s="132">
         <f>IF(A10="","",SUM($G$5:G10))</f>
         <v/>
       </c>
-      <c r="M10" s="160">
+      <c r="M10" s="132">
         <f>IF(A10="","",SUM($H$5:H10))</f>
         <v/>
       </c>
-      <c r="N10" s="217">
-        <f>IF(A10="","",J10+K10+L10+M10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="109">
-      <c r="A11" s="165" t="n"/>
-      <c r="B11" s="169" t="n"/>
-      <c r="C11" s="165" t="n"/>
-      <c r="D11" s="212" t="n"/>
-      <c r="E11" s="166" t="n"/>
-      <c r="F11" s="166" t="n"/>
-      <c r="G11" s="166" t="n"/>
-      <c r="H11" s="166" t="n"/>
-      <c r="I11" s="213">
-        <f>IF(A11="","",SUM(E11:H11))</f>
-        <v/>
-      </c>
-      <c r="J11" s="154">
-        <f>IF(A11="","",SUM($E$5:E11))</f>
-        <v/>
-      </c>
-      <c r="K11" s="154">
-        <f>IF(A11="","",SUM($F$5:F11))</f>
-        <v/>
-      </c>
-      <c r="L11" s="154">
+      <c r="N10" s="132">
+        <f>IF(A10="","",SUM($I$5:I10))</f>
+        <v/>
+      </c>
+      <c r="O10" s="132">
+        <f>IF(A10="","",SUM($J$5:J10))</f>
+        <v/>
+      </c>
+      <c r="P10" s="132">
+        <f>IF(A10="","",L10+M10+N10+O10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="128" t="n"/>
+      <c r="B11" s="202" t="n"/>
+      <c r="C11" s="128" t="n"/>
+      <c r="D11" s="128" t="n"/>
+      <c r="E11" s="128" t="n"/>
+      <c r="F11" s="128" t="n"/>
+      <c r="G11" s="131" t="n"/>
+      <c r="H11" s="131" t="n"/>
+      <c r="I11" s="131" t="n"/>
+      <c r="J11" s="131" t="n"/>
+      <c r="K11" s="132">
+        <f>IF(A11="","",SUM(G11:J11))</f>
+        <v/>
+      </c>
+      <c r="L11" s="132">
         <f>IF(A11="","",SUM($G$5:G11))</f>
         <v/>
       </c>
-      <c r="M11" s="154">
+      <c r="M11" s="132">
         <f>IF(A11="","",SUM($H$5:H11))</f>
         <v/>
       </c>
-      <c r="N11" s="214">
-        <f>IF(A11="","",J11+K11+L11+M11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="109">
-      <c r="A12" s="172" t="n"/>
-      <c r="B12" s="176" t="n"/>
-      <c r="C12" s="172" t="n"/>
-      <c r="D12" s="215" t="n"/>
-      <c r="E12" s="173" t="n"/>
-      <c r="F12" s="173" t="n"/>
-      <c r="G12" s="173" t="n"/>
-      <c r="H12" s="173" t="n"/>
-      <c r="I12" s="216">
-        <f>IF(A12="","",SUM(E12:H12))</f>
-        <v/>
-      </c>
-      <c r="J12" s="160">
-        <f>IF(A12="","",SUM($E$5:E12))</f>
-        <v/>
-      </c>
-      <c r="K12" s="160">
-        <f>IF(A12="","",SUM($F$5:F12))</f>
-        <v/>
-      </c>
-      <c r="L12" s="160">
+      <c r="N11" s="132">
+        <f>IF(A11="","",SUM($I$5:I11))</f>
+        <v/>
+      </c>
+      <c r="O11" s="132">
+        <f>IF(A11="","",SUM($J$5:J11))</f>
+        <v/>
+      </c>
+      <c r="P11" s="132">
+        <f>IF(A11="","",L11+M11+N11+O11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="128" t="n"/>
+      <c r="B12" s="202" t="n"/>
+      <c r="C12" s="128" t="n"/>
+      <c r="D12" s="128" t="n"/>
+      <c r="E12" s="128" t="n"/>
+      <c r="F12" s="128" t="n"/>
+      <c r="G12" s="131" t="n"/>
+      <c r="H12" s="131" t="n"/>
+      <c r="I12" s="131" t="n"/>
+      <c r="J12" s="131" t="n"/>
+      <c r="K12" s="132">
+        <f>IF(A12="","",SUM(G12:J12))</f>
+        <v/>
+      </c>
+      <c r="L12" s="132">
         <f>IF(A12="","",SUM($G$5:G12))</f>
         <v/>
       </c>
-      <c r="M12" s="160">
+      <c r="M12" s="132">
         <f>IF(A12="","",SUM($H$5:H12))</f>
         <v/>
       </c>
-      <c r="N12" s="217">
-        <f>IF(A12="","",J12+K12+L12+M12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="109">
-      <c r="A13" s="165" t="n"/>
-      <c r="B13" s="169" t="n"/>
-      <c r="C13" s="165" t="n"/>
-      <c r="D13" s="212" t="n"/>
-      <c r="E13" s="166" t="n"/>
-      <c r="F13" s="166" t="n"/>
-      <c r="G13" s="166" t="n"/>
-      <c r="H13" s="166" t="n"/>
-      <c r="I13" s="213">
-        <f>IF(A13="","",SUM(E13:H13))</f>
-        <v/>
-      </c>
-      <c r="J13" s="154">
-        <f>IF(A13="","",SUM($E$5:E13))</f>
-        <v/>
-      </c>
-      <c r="K13" s="154">
-        <f>IF(A13="","",SUM($F$5:F13))</f>
-        <v/>
-      </c>
-      <c r="L13" s="154">
+      <c r="N12" s="132">
+        <f>IF(A12="","",SUM($I$5:I12))</f>
+        <v/>
+      </c>
+      <c r="O12" s="132">
+        <f>IF(A12="","",SUM($J$5:J12))</f>
+        <v/>
+      </c>
+      <c r="P12" s="132">
+        <f>IF(A12="","",L12+M12+N12+O12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="128" t="n"/>
+      <c r="B13" s="202" t="n"/>
+      <c r="C13" s="128" t="n"/>
+      <c r="D13" s="128" t="n"/>
+      <c r="E13" s="128" t="n"/>
+      <c r="F13" s="128" t="n"/>
+      <c r="G13" s="131" t="n"/>
+      <c r="H13" s="131" t="n"/>
+      <c r="I13" s="131" t="n"/>
+      <c r="J13" s="131" t="n"/>
+      <c r="K13" s="132">
+        <f>IF(A13="","",SUM(G13:J13))</f>
+        <v/>
+      </c>
+      <c r="L13" s="132">
         <f>IF(A13="","",SUM($G$5:G13))</f>
         <v/>
       </c>
-      <c r="M13" s="154">
+      <c r="M13" s="132">
         <f>IF(A13="","",SUM($H$5:H13))</f>
         <v/>
       </c>
-      <c r="N13" s="214">
-        <f>IF(A13="","",J13+K13+L13+M13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="109">
-      <c r="A14" s="172" t="n"/>
-      <c r="B14" s="176" t="n"/>
-      <c r="C14" s="172" t="n"/>
-      <c r="D14" s="215" t="n"/>
-      <c r="E14" s="173" t="n"/>
-      <c r="F14" s="173" t="n"/>
-      <c r="G14" s="173" t="n"/>
-      <c r="H14" s="173" t="n"/>
-      <c r="I14" s="216">
-        <f>IF(A14="","",SUM(E14:H14))</f>
-        <v/>
-      </c>
-      <c r="J14" s="160">
-        <f>IF(A14="","",SUM($E$5:E14))</f>
-        <v/>
-      </c>
-      <c r="K14" s="160">
-        <f>IF(A14="","",SUM($F$5:F14))</f>
-        <v/>
-      </c>
-      <c r="L14" s="160">
+      <c r="N13" s="132">
+        <f>IF(A13="","",SUM($I$5:I13))</f>
+        <v/>
+      </c>
+      <c r="O13" s="132">
+        <f>IF(A13="","",SUM($J$5:J13))</f>
+        <v/>
+      </c>
+      <c r="P13" s="132">
+        <f>IF(A13="","",L13+M13+N13+O13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="128" t="n"/>
+      <c r="B14" s="202" t="n"/>
+      <c r="C14" s="128" t="n"/>
+      <c r="D14" s="128" t="n"/>
+      <c r="E14" s="128" t="n"/>
+      <c r="F14" s="128" t="n"/>
+      <c r="G14" s="131" t="n"/>
+      <c r="H14" s="131" t="n"/>
+      <c r="I14" s="131" t="n"/>
+      <c r="J14" s="131" t="n"/>
+      <c r="K14" s="132">
+        <f>IF(A14="","",SUM(G14:J14))</f>
+        <v/>
+      </c>
+      <c r="L14" s="132">
         <f>IF(A14="","",SUM($G$5:G14))</f>
         <v/>
       </c>
-      <c r="M14" s="160">
+      <c r="M14" s="132">
         <f>IF(A14="","",SUM($H$5:H14))</f>
         <v/>
       </c>
-      <c r="N14" s="217">
-        <f>IF(A14="","",J14+K14+L14+M14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="109">
-      <c r="A17" s="115" t="inlineStr">
+      <c r="N14" s="132">
+        <f>IF(A14="","",SUM($I$5:I14))</f>
+        <v/>
+      </c>
+      <c r="O14" s="132">
+        <f>IF(A14="","",SUM($J$5:J14))</f>
+        <v/>
+      </c>
+      <c r="P14" s="132">
+        <f>IF(A14="","",L14+M14+N14+O14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="123" t="inlineStr">
         <is>
           <t>CLIN Funding Status (auto — reads Projects tab, not this log)</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="27.75" customHeight="1" s="109">
-      <c r="A18" s="151" t="inlineStr">
+    <row r="17" ht="28" customHeight="1" s="109">
+      <c r="A17" s="137" t="inlineStr">
         <is>
           <t>CLIN</t>
         </is>
       </c>
-      <c r="B18" s="151" t="inlineStr">
-        <is>
-          <t>Cumulative
-TOA $</t>
-        </is>
-      </c>
-      <c r="C18" s="151" t="inlineStr">
+      <c r="B17" s="137" t="inlineStr">
+        <is>
+          <t>Funded $
+(from Projects)</t>
+        </is>
+      </c>
+      <c r="C17" s="137" t="inlineStr">
+        <is>
+          <t>Mod Log
+Total $</t>
+        </is>
+      </c>
+      <c r="D17" s="137" t="inlineStr">
+        <is>
+          <t>Reconciled?</t>
+        </is>
+      </c>
+      <c r="E17" s="137" t="inlineStr">
         <is>
           <t>Spent to
 Date $</t>
         </is>
       </c>
-      <c r="D18" s="151" t="inlineStr">
+      <c r="F17" s="137" t="inlineStr">
         <is>
           <t>Remaining
 $</t>
         </is>
       </c>
-      <c r="E18" s="151" t="inlineStr">
+      <c r="G17" s="137" t="inlineStr">
         <is>
           <t>% Used</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="109">
-      <c r="A19" s="218" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="127" t="inlineStr">
         <is>
           <t>Labor</t>
         </is>
       </c>
-      <c r="B19" s="154">
+      <c r="B18" s="132">
         <f>SUM(Projects!$C$6:$C$13)</f>
         <v/>
       </c>
-      <c r="C19" s="155">
+      <c r="C18" s="132">
+        <f>SUM(G$5:G$14)</f>
+        <v/>
+      </c>
+      <c r="D18" s="138">
+        <f>IF(ROUND(B18-C18,2)=0,"Match","MISMATCH: "&amp;TEXT(C18-B18,"+$#,##0;-$#,##0"))</f>
+        <v/>
+      </c>
+      <c r="E18" s="132">
         <f>SUM(Dashboard!$D$21:$D$32)</f>
         <v/>
       </c>
-      <c r="D19" s="154">
-        <f>B19-C19</f>
-        <v/>
-      </c>
-      <c r="E19" s="157">
-        <f>IFERROR(C19/B19,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="109">
-      <c r="A20" s="219" t="inlineStr">
+      <c r="F18" s="132">
+        <f>B18-E18</f>
+        <v/>
+      </c>
+      <c r="G18" s="129">
+        <f>IFERROR(E18/B18,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="127" t="inlineStr">
         <is>
           <t>Travel</t>
         </is>
       </c>
-      <c r="B20" s="160">
+      <c r="B19" s="132">
         <f>SUM(Projects!$D$6:$D$13)</f>
         <v/>
       </c>
-      <c r="C20" s="161">
+      <c r="C19" s="132">
+        <f>SUM(H$5:H$14)</f>
+        <v/>
+      </c>
+      <c r="D19" s="138">
+        <f>IF(ROUND(B19-C19,2)=0,"Match","MISMATCH: "&amp;TEXT(C19-B19,"+$#,##0;-$#,##0"))</f>
+        <v/>
+      </c>
+      <c r="E19" s="132">
         <f>SUM(Dashboard!$G$21:$G$32)</f>
         <v/>
       </c>
-      <c r="D20" s="160">
-        <f>B20-C20</f>
-        <v/>
-      </c>
-      <c r="E20" s="163">
-        <f>IFERROR(C20/B20,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="15" customHeight="1" s="109">
-      <c r="A21" s="218" t="inlineStr">
+      <c r="F19" s="132">
+        <f>B19-E19</f>
+        <v/>
+      </c>
+      <c r="G19" s="129">
+        <f>IFERROR(E19/B19,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="127" t="inlineStr">
         <is>
           <t>ODC</t>
         </is>
       </c>
-      <c r="B21" s="154">
+      <c r="B20" s="132">
         <f>SUM(Projects!$E$6:$E$13)</f>
         <v/>
       </c>
-      <c r="C21" s="155">
+      <c r="C20" s="132">
+        <f>SUM(I$5:I$14)</f>
+        <v/>
+      </c>
+      <c r="D20" s="138">
+        <f>IF(ROUND(B20-C20,2)=0,"Match","MISMATCH: "&amp;TEXT(C20-B20,"+$#,##0;-$#,##0"))</f>
+        <v/>
+      </c>
+      <c r="E20" s="132">
         <f>SUM(Dashboard!$E$21:$E$32)</f>
         <v/>
       </c>
-      <c r="D21" s="154">
-        <f>B21-C21</f>
-        <v/>
-      </c>
-      <c r="E21" s="157">
-        <f>IFERROR(C21/B21,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" ht="15" customHeight="1" s="109">
-      <c r="A22" s="219" t="inlineStr">
+      <c r="F20" s="132">
+        <f>B20-E20</f>
+        <v/>
+      </c>
+      <c r="G20" s="129">
+        <f>IFERROR(E20/B20,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="127" t="inlineStr">
         <is>
           <t>M&amp;E</t>
         </is>
       </c>
-      <c r="B22" s="160">
+      <c r="B21" s="132">
         <f>SUM(Projects!$F$6:$F$13)</f>
         <v/>
       </c>
-      <c r="C22" s="161">
+      <c r="C21" s="132">
+        <f>SUM(J$5:J$14)</f>
+        <v/>
+      </c>
+      <c r="D21" s="138">
+        <f>IF(ROUND(B21-C21,2)=0,"Match","MISMATCH: "&amp;TEXT(C21-B21,"+$#,##0;-$#,##0"))</f>
+        <v/>
+      </c>
+      <c r="E21" s="132">
         <f>SUM(Dashboard!$F$21:$F$32)</f>
         <v/>
       </c>
-      <c r="D22" s="160">
-        <f>B22-C22</f>
-        <v/>
-      </c>
-      <c r="E22" s="163">
-        <f>IFERROR(C22/B22,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="109">
-      <c r="A23" s="220" t="inlineStr">
+      <c r="F21" s="132">
+        <f>B21-E21</f>
+        <v/>
+      </c>
+      <c r="G21" s="129">
+        <f>IFERROR(E21/B21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="124" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B23" s="221">
-        <f>SUM(B19:B22)</f>
-        <v/>
-      </c>
-      <c r="C23" s="221">
-        <f>SUM(C19:C22)</f>
-        <v/>
-      </c>
-      <c r="D23" s="221">
-        <f>SUM(D19:D22)</f>
-        <v/>
-      </c>
-      <c r="E23" s="222">
-        <f>IFERROR(C23/B23,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" ht="15" customHeight="1" s="109">
-      <c r="A26" s="111" t="inlineStr">
+      <c r="B22" s="135">
+        <f>SUM(B18:B21)</f>
+        <v/>
+      </c>
+      <c r="C22" s="135">
+        <f>SUM(C18:C21)</f>
+        <v/>
+      </c>
+      <c r="D22" s="139">
+        <f>IF(ROUND(B22-C22,2)=0,"Match","MISMATCH: "&amp;TEXT(C22-B22,"+$#,##0;-$#,##0"))</f>
+        <v/>
+      </c>
+      <c r="E22" s="135">
+        <f>SUM(E18:E21)</f>
+        <v/>
+      </c>
+      <c r="F22" s="135">
+        <f>SUM(F18:F21)</f>
+        <v/>
+      </c>
+      <c r="G22" s="140">
+        <f>IFERROR(E22/B22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1" s="109">
+      <c r="A24" s="114" t="inlineStr">
+        <is>
+          <t>Reconciled = this log's CLIN totals match what's actually funded on the Projects tab. If it says MISMATCH, someone updated one tab without the other — fix Projects (the source of truth) or log the missing mod here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="117" t="inlineStr">
         <is>
           <t>Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A3:N3"/>
+  <autoFilter ref="A4:P14"/>
+  <mergeCells count="2">
+    <mergeCell ref="A24:P24"/>
+    <mergeCell ref="A3:P3"/>
   </mergeCells>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <conditionalFormatting sqref="D18">
+    <cfRule type="expression" priority="1" dxfId="14">
+      <formula>D18="Match"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="11">
+      <formula>D18&lt;&gt;"Match"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D19">
+    <cfRule type="expression" priority="3" dxfId="14">
+      <formula>D19="Match"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="11">
+      <formula>D19&lt;&gt;"Match"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D20">
+    <cfRule type="expression" priority="5" dxfId="14">
+      <formula>D20="Match"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="11">
+      <formula>D20&lt;&gt;"Match"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D21">
+    <cfRule type="expression" priority="7" dxfId="14">
+      <formula>D21="Match"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="11">
+      <formula>D21&lt;&gt;"Match"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D22">
+    <cfRule type="expression" priority="9" dxfId="15">
+      <formula>D22="Match"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="16">
+      <formula>D22&lt;&gt;"Match"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="F5:F14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Projects!$A$6:$A$13</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -8531,14 +8668,14 @@
       </c>
     </row>
     <row r="3" ht="27.75" customHeight="1" s="109">
-      <c r="A3" s="223" t="inlineStr">
+      <c r="A3" s="210" t="inlineStr">
         <is>
           <t>Quick answer for "what would it cost to add or change this person?" — a standalone what-if, separate from your actual Labor log. Doesn't affect Dashboard totals or Labor actuals.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="109">
-      <c r="A5" s="224" t="inlineStr">
+      <c r="A5" s="211" t="inlineStr">
         <is>
           <t>SCENARIO INPUTS</t>
         </is>
@@ -8552,105 +8689,105 @@
       </c>
     </row>
     <row r="8" ht="19.5" customHeight="1" s="109">
-      <c r="A8" s="218" t="inlineStr">
+      <c r="A8" s="212" t="inlineStr">
         <is>
           <t>Role / LCAT</t>
         </is>
       </c>
-      <c r="B8" s="225" t="inlineStr">
+      <c r="B8" s="213" t="inlineStr">
         <is>
           <t>Engineer 4</t>
         </is>
       </c>
-      <c r="C8" s="226" t="n"/>
-      <c r="D8" s="226" t="n"/>
-      <c r="E8" s="226" t="n"/>
+      <c r="C8" s="214" t="n"/>
+      <c r="D8" s="214" t="n"/>
+      <c r="E8" s="214" t="n"/>
     </row>
     <row r="9" ht="19.5" customHeight="1" s="109">
-      <c r="A9" s="218" t="inlineStr">
+      <c r="A9" s="212" t="inlineStr">
         <is>
           <t>Employee Type</t>
         </is>
       </c>
-      <c r="B9" s="225" t="inlineStr">
+      <c r="B9" s="213" t="inlineStr">
         <is>
           <t>Exempt</t>
         </is>
       </c>
-      <c r="C9" s="226" t="n"/>
-      <c r="D9" s="226" t="n"/>
-      <c r="E9" s="226" t="n"/>
+      <c r="C9" s="214" t="n"/>
+      <c r="D9" s="214" t="n"/>
+      <c r="E9" s="214" t="n"/>
     </row>
     <row r="10" ht="19.5" customHeight="1" s="109">
-      <c r="A10" s="218" t="inlineStr">
+      <c r="A10" s="212" t="inlineStr">
         <is>
           <t>Annual Salary (Exempt only)</t>
         </is>
       </c>
-      <c r="B10" s="227" t="n">
+      <c r="B10" s="215" t="n">
         <v>150000</v>
       </c>
-      <c r="C10" s="226" t="n"/>
-      <c r="D10" s="226" t="n"/>
-      <c r="E10" s="226" t="n"/>
+      <c r="C10" s="214" t="n"/>
+      <c r="D10" s="214" t="n"/>
+      <c r="E10" s="214" t="n"/>
     </row>
     <row r="11" ht="19.5" customHeight="1" s="109">
-      <c r="A11" s="218" t="inlineStr">
+      <c r="A11" s="212" t="inlineStr">
         <is>
           <t>Direct Hourly Rate (Non-Exempt only)</t>
         </is>
       </c>
-      <c r="B11" s="228" t="n"/>
-      <c r="C11" s="226" t="n"/>
-      <c r="D11" s="226" t="n"/>
-      <c r="E11" s="226" t="n"/>
+      <c r="B11" s="216" t="n"/>
+      <c r="C11" s="214" t="n"/>
+      <c r="D11" s="214" t="n"/>
+      <c r="E11" s="214" t="n"/>
     </row>
     <row r="12" ht="19.5" customHeight="1" s="109">
-      <c r="A12" s="218" t="inlineStr">
+      <c r="A12" s="212" t="inlineStr">
         <is>
           <t>Standard Annual Hours</t>
         </is>
       </c>
-      <c r="B12" s="225" t="n">
+      <c r="B12" s="213" t="n">
         <v>2080</v>
       </c>
-      <c r="C12" s="226" t="n"/>
-      <c r="D12" s="226" t="n"/>
-      <c r="E12" s="226" t="n"/>
+      <c r="C12" s="214" t="n"/>
+      <c r="D12" s="214" t="n"/>
+      <c r="E12" s="214" t="n"/>
     </row>
     <row r="13" ht="19.5" customHeight="1" s="109">
-      <c r="A13" s="218" t="inlineStr">
+      <c r="A13" s="212" t="inlineStr">
         <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="B13" s="229" t="n">
+      <c r="B13" s="217" t="n">
         <v>46266</v>
       </c>
-      <c r="C13" s="226" t="n"/>
-      <c r="D13" s="226" t="n"/>
-      <c r="E13" s="226" t="n"/>
+      <c r="C13" s="214" t="n"/>
+      <c r="D13" s="214" t="n"/>
+      <c r="E13" s="214" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="109">
-      <c r="A14" s="218" t="inlineStr">
+      <c r="A14" s="212" t="inlineStr">
         <is>
           <t>End Date</t>
         </is>
       </c>
-      <c r="B14" s="230">
+      <c r="B14" s="218">
         <f>Dashboard!$C$6</f>
         <v/>
       </c>
-      <c r="C14" s="231" t="inlineStr">
+      <c r="C14" s="219" t="inlineStr">
         <is>
           <t>Defaults to your PoP End on Dashboard — type over it for a custom end date.</t>
         </is>
       </c>
-      <c r="D14" s="232" t="n"/>
-      <c r="E14" s="233" t="n"/>
+      <c r="D14" s="220" t="n"/>
+      <c r="E14" s="221" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="109">
-      <c r="A16" s="224" t="inlineStr">
+      <c r="A16" s="211" t="inlineStr">
         <is>
           <t>BASE LABOR COST (auto)</t>
         </is>
@@ -8664,7 +8801,7 @@
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="109">
-      <c r="A19" s="234" t="inlineStr">
+      <c r="A19" s="222" t="inlineStr">
         <is>
           <t>Straight-Time Rate $/hr</t>
         </is>
@@ -8673,26 +8810,26 @@
         <f>IF(B9="Exempt",IF(B12=0,"",B10/B12),B11)</f>
         <v/>
       </c>
-      <c r="C19" s="226" t="n"/>
-      <c r="D19" s="226" t="n"/>
-      <c r="E19" s="226" t="n"/>
+      <c r="C19" s="214" t="n"/>
+      <c r="D19" s="214" t="n"/>
+      <c r="E19" s="214" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="109">
-      <c r="A20" s="234" t="inlineStr">
+      <c r="A20" s="222" t="inlineStr">
         <is>
           <t>Days in Period</t>
         </is>
       </c>
-      <c r="B20" s="235">
+      <c r="B20" s="223">
         <f>IF(OR(B13="",B14=""),"",B14-B13+1)</f>
         <v/>
       </c>
-      <c r="C20" s="226" t="n"/>
-      <c r="D20" s="226" t="n"/>
-      <c r="E20" s="226" t="n"/>
+      <c r="C20" s="214" t="n"/>
+      <c r="D20" s="214" t="n"/>
+      <c r="E20" s="214" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="109">
-      <c r="A21" s="234" t="inlineStr">
+      <c r="A21" s="222" t="inlineStr">
         <is>
           <t>Estimated Hours in Period</t>
         </is>
@@ -8701,12 +8838,12 @@
         <f>IF(B20="","",B12*B20/365)</f>
         <v/>
       </c>
-      <c r="C21" s="226" t="n"/>
-      <c r="D21" s="226" t="n"/>
-      <c r="E21" s="226" t="n"/>
+      <c r="C21" s="214" t="n"/>
+      <c r="D21" s="214" t="n"/>
+      <c r="E21" s="214" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="109">
-      <c r="A22" s="234" t="inlineStr">
+      <c r="A22" s="222" t="inlineStr">
         <is>
           <t>Direct Labor $</t>
         </is>
@@ -8715,12 +8852,12 @@
         <f>IF(OR(B21="",B19=""),"",B21*B19)</f>
         <v/>
       </c>
-      <c r="C22" s="226" t="n"/>
-      <c r="D22" s="226" t="n"/>
-      <c r="E22" s="226" t="n"/>
+      <c r="C22" s="214" t="n"/>
+      <c r="D22" s="214" t="n"/>
+      <c r="E22" s="214" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1" s="109">
-      <c r="A23" s="234" t="inlineStr">
+      <c r="A23" s="222" t="inlineStr">
         <is>
           <t>Fringe $</t>
         </is>
@@ -8729,12 +8866,12 @@
         <f>IF(B22="","",B22*Rates!$B$6)</f>
         <v/>
       </c>
-      <c r="C23" s="226" t="n"/>
-      <c r="D23" s="226" t="n"/>
-      <c r="E23" s="226" t="n"/>
+      <c r="C23" s="214" t="n"/>
+      <c r="D23" s="214" t="n"/>
+      <c r="E23" s="214" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="109">
-      <c r="A24" s="234" t="inlineStr">
+      <c r="A24" s="222" t="inlineStr">
         <is>
           <t>OH $</t>
         </is>
@@ -8743,26 +8880,26 @@
         <f>IF(B22="","",(B22+B23)*Rates!$B$7)</f>
         <v/>
       </c>
-      <c r="C24" s="226" t="n"/>
-      <c r="D24" s="226" t="n"/>
-      <c r="E24" s="226" t="n"/>
+      <c r="C24" s="214" t="n"/>
+      <c r="D24" s="214" t="n"/>
+      <c r="E24" s="214" t="n"/>
     </row>
     <row r="25" ht="25.5" customHeight="1" s="109">
-      <c r="A25" s="236" t="inlineStr">
+      <c r="A25" s="224" t="inlineStr">
         <is>
           <t>Base Fully Burdened Labor $</t>
         </is>
       </c>
-      <c r="B25" s="237">
+      <c r="B25" s="225">
         <f>IF(B22="","",B22+B23+B24)</f>
         <v/>
       </c>
-      <c r="C25" s="238" t="n"/>
-      <c r="D25" s="238" t="n"/>
-      <c r="E25" s="238" t="n"/>
+      <c r="C25" s="226" t="n"/>
+      <c r="D25" s="226" t="n"/>
+      <c r="E25" s="226" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="109">
-      <c r="A27" s="224" t="inlineStr">
+      <c r="A27" s="211" t="inlineStr">
         <is>
           <t>LOCATION / ALLOWANCE ADDERS</t>
         </is>
@@ -8872,20 +9009,20 @@
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="109">
-      <c r="A35" s="220" t="inlineStr">
+      <c r="A35" s="227" t="inlineStr">
         <is>
           <t>Total Adders</t>
         </is>
       </c>
-      <c r="B35" s="238" t="n"/>
-      <c r="C35" s="238" t="n"/>
-      <c r="D35" s="221">
+      <c r="B35" s="226" t="n"/>
+      <c r="C35" s="226" t="n"/>
+      <c r="D35" s="228">
         <f>SUM(D31:D34)</f>
         <v/>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="109">
-      <c r="A37" s="224" t="inlineStr">
+      <c r="A37" s="211" t="inlineStr">
         <is>
           <t>ROM ESTIMATE</t>
         </is>
@@ -8899,7 +9036,7 @@
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="109">
-      <c r="A40" s="234" t="inlineStr">
+      <c r="A40" s="222" t="inlineStr">
         <is>
           <t>Subtotal (Labor + Adders) $</t>
         </is>
@@ -8908,12 +9045,12 @@
         <f>IF(B25="","",B25+D35)</f>
         <v/>
       </c>
-      <c r="C40" s="226" t="n"/>
-      <c r="D40" s="226" t="n"/>
-      <c r="E40" s="226" t="n"/>
+      <c r="C40" s="214" t="n"/>
+      <c r="D40" s="214" t="n"/>
+      <c r="E40" s="214" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1" s="109">
-      <c r="A41" s="234" t="inlineStr">
+      <c r="A41" s="222" t="inlineStr">
         <is>
           <t>G&amp;A $</t>
         </is>
@@ -8922,12 +9059,12 @@
         <f>IF(B40="","",B40*Rates!$B$8)</f>
         <v/>
       </c>
-      <c r="C41" s="226" t="n"/>
-      <c r="D41" s="226" t="n"/>
-      <c r="E41" s="226" t="n"/>
+      <c r="C41" s="214" t="n"/>
+      <c r="D41" s="214" t="n"/>
+      <c r="E41" s="214" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="109">
-      <c r="A42" s="234" t="inlineStr">
+      <c r="A42" s="222" t="inlineStr">
         <is>
           <t>Total Cost $</t>
         </is>
@@ -8936,12 +9073,12 @@
         <f>IF(B40="","",B40+B41)</f>
         <v/>
       </c>
-      <c r="C42" s="226" t="n"/>
-      <c r="D42" s="226" t="n"/>
-      <c r="E42" s="226" t="n"/>
+      <c r="C42" s="214" t="n"/>
+      <c r="D42" s="214" t="n"/>
+      <c r="E42" s="214" t="n"/>
     </row>
     <row r="43" ht="15" customHeight="1" s="109">
-      <c r="A43" s="234" t="inlineStr">
+      <c r="A43" s="222" t="inlineStr">
         <is>
           <t>Fee $</t>
         </is>
@@ -8950,26 +9087,26 @@
         <f>IF(B42="","",B42*Rates!$C$18)</f>
         <v/>
       </c>
-      <c r="C43" s="226" t="n"/>
-      <c r="D43" s="226" t="n"/>
-      <c r="E43" s="226" t="n"/>
+      <c r="C43" s="214" t="n"/>
+      <c r="D43" s="214" t="n"/>
+      <c r="E43" s="214" t="n"/>
     </row>
     <row r="44" ht="30" customHeight="1" s="109">
-      <c r="A44" s="239" t="inlineStr">
+      <c r="A44" s="229" t="inlineStr">
         <is>
           <t>TOTAL ROM ESTIMATE (fully burdened)</t>
         </is>
       </c>
-      <c r="B44" s="240">
+      <c r="B44" s="230">
         <f>IF(B42="","",B42+B43)</f>
         <v/>
       </c>
-      <c r="C44" s="238" t="n"/>
-      <c r="D44" s="238" t="n"/>
-      <c r="E44" s="238" t="n"/>
+      <c r="C44" s="226" t="n"/>
+      <c r="D44" s="226" t="n"/>
+      <c r="E44" s="226" t="n"/>
     </row>
     <row r="46" ht="24" customHeight="1" s="109">
-      <c r="A46" s="241">
+      <c r="A46" s="231">
         <f>"For "&amp;B8&amp;" from "&amp;TEXT(B13,"mm/dd/yyyy")&amp;" to "&amp;TEXT(B14,"mm/dd/yyyy")&amp;" ("&amp;B20&amp;" days): "&amp;TEXT(B44,"$#,##0")&amp;" fully burdened, ROM estimate."</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Rates tab: add CR (Cost Reimbursable) fee type for cost-only CLINs
- Fee Type dropdown now offers Fixed / Award / CR
- CR resolves to 0% fee rate, for CLINs that earn no fee at all
- Travel now defaults to CR in the shipped sample (was Fixed)
- Updated Fee Structure note text to explain CR
</commit_message>
<xml_diff>
--- a/client/public/examples/cost-and-burn-rate-tracker.xlsx
+++ b/client/public/examples/cost-and-burn-rate-tracker.xlsx
@@ -9268,7 +9268,7 @@
     <row r="11" ht="28" customHeight="1" s="109">
       <c r="A11" s="117" t="inlineStr">
         <is>
-          <t>Fixed = flat % of Total Cost (CPFF). Award = pool rate, actual earned fee depends on your award fee score. A contract can run BOTH — pick which CLINs draw from which pool in the table below.</t>
+          <t>Fixed = flat % of Total Cost (CPFF). Award = pool rate, actual earned fee depends on your award fee score. CR = Cost Reimbursable — no fee at all (0%), common for cost-only CLINs like travel. A contract can run all three — pick which CLINs draw from which pool in the table below.</t>
         </is>
       </c>
     </row>
@@ -9335,7 +9335,7 @@
         </is>
       </c>
       <c r="C18" s="129">
-        <f>IF(B18="Fixed",$B$13,IF(B18="Award",$B$14,NA()))</f>
+        <f>IF(B18="Fixed",$B$13,IF(B18="Award",$B$14,IF(B18="CR",0,NA())))</f>
         <v/>
       </c>
     </row>
@@ -9347,11 +9347,11 @@
       </c>
       <c r="B19" s="128" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C19" s="129">
-        <f>IF(B19="Fixed",$B$13,IF(B19="Award",$B$14,NA()))</f>
+        <f>IF(B19="Fixed",$B$13,IF(B19="Award",$B$14,IF(B19="CR",0,NA())))</f>
         <v/>
       </c>
     </row>
@@ -9367,7 +9367,7 @@
         </is>
       </c>
       <c r="C20" s="129">
-        <f>IF(B20="Fixed",$B$13,IF(B20="Award",$B$14,NA()))</f>
+        <f>IF(B20="Fixed",$B$13,IF(B20="Award",$B$14,IF(B20="CR",0,NA())))</f>
         <v/>
       </c>
     </row>
@@ -9383,14 +9383,14 @@
         </is>
       </c>
       <c r="C21" s="129">
-        <f>IF(B21="Fixed",$B$13,IF(B21="Award",$B$14,NA()))</f>
+        <f>IF(B21="Fixed",$B$13,IF(B21="Award",$B$14,IF(B21="CR",0,NA())))</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1" s="109">
       <c r="A23" s="117" t="inlineStr">
         <is>
-          <t>This is what Dashboard, Revenue Forecast, and the ROM Calculator (Labor row) use — Total Cost per CLIN times that CLIN's Applicable Fee Rate.</t>
+          <t>This is what Dashboard, Revenue Forecast, and the ROM Calculator (Labor row) use — Total Cost per CLIN times that CLIN's Applicable Fee Rate. CR CLINs always resolve to 0%.</t>
         </is>
       </c>
     </row>
@@ -9415,7 +9415,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="B18 B19 B20 B21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Fixed,Award"</formula1>
+      <formula1>"Fixed,Award,CR"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add license watermark + password protection for resale
- Hidden (veryHidden) _License sheet: fill in Licensed To / Email before sending
  a sold copy. Every tab's footer picks it up automatically ('Licensed to: X'),
  so leaked copies are traceable back to the buyer.
- Document metadata set: creator/company Acqlerate, title, and a copyright/
  license description in the file properties.
- Every sheet password-protected (formulas and formatting locked); every
  blue-font 'your input' cell — the workbook's own existing color convention —
  stays fully editable. AutoFilter and sort remain usable on the item logs.
  Workbook structure locked too (can't add/remove/reorder/unhide sheets).
  Password: Acqlerate-2026 (native Excel protection — deterrent, not a vault;
  see chat for the full explanation of what this does and doesn't stop).
</commit_message>
<xml_diff>
--- a/client/public/examples/cost-and-burn-rate-tracker.xlsx
+++ b/client/public/examples/cost-and-burn-rate-tracker.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
+  <workbookProtection workbookPassword="B0B1" lockStructure="1"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
@@ -21,6 +21,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Burn Rate Forecast" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FundingMods" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROM Calculator" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_License" sheetId="15" state="veryHidden" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Projects'!$A$4:$G$13</definedName>
@@ -48,7 +49,7 @@
     <numFmt numFmtId="172" formatCode="m/d/yyyy"/>
     <numFmt numFmtId="173" formatCode="0.00&quot;x&quot;"/>
   </numFmts>
-  <fonts count="35">
+  <fonts count="36">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -209,6 +210,11 @@
       <i val="1"/>
       <color rgb="FF0F172A"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -575,7 +581,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="228">
+  <cellXfs count="230">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -910,70 +916,78 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="26" fillId="11" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="27" fillId="11" borderId="14" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="12" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="28" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="14" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="9" fontId="29" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="26" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="28" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="27" fillId="0" borderId="14" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="29" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="25" fillId="13" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="26" fillId="13" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="25" fillId="13" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="26" fillId="13" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="10" fillId="2" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
@@ -1014,7 +1028,7 @@
     <xf numFmtId="164" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="166" fontId="30" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="31" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1036,112 +1050,148 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="169" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="14" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="169" fontId="31" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="173" fontId="29" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="169" fontId="30" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="170" fontId="10" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="173" fontId="28" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="170" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="170" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="10" fillId="6" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="10" fillId="6" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="169" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="10" fillId="6" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="6" borderId="14" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="169" fontId="31" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="173" fontId="29" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="169" fontId="30" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="170" fontId="10" fillId="6" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="173" fontId="28" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="170" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="170" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="12" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="26" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="26" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="28" fillId="13" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="27" fillId="0" borderId="14" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="170" fontId="27" fillId="0" borderId="15" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="170" fontId="29" fillId="13" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="28" fillId="15" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="26" fillId="15" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="28" fillId="15" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="28" fillId="16" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="26" fillId="16" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="28" fillId="16" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="28" fillId="17" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="26" fillId="17" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="28" fillId="17" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="28" fillId="18" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="26" fillId="18" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="28" fillId="18" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="28" fillId="13" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="17" fontId="28" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="172" fontId="26" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="25" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="23" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="23" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="29" fillId="15" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="27" fillId="15" borderId="14" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="29" fillId="15" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="29" fillId="16" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="27" fillId="16" borderId="14" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="29" fillId="16" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="29" fillId="17" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="27" fillId="17" borderId="14" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="29" fillId="17" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="29" fillId="18" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="27" fillId="18" borderId="14" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="29" fillId="18" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="29" fillId="13" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="17" fontId="29" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="27" fillId="0" borderId="14" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="24" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="24" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="28" fillId="19" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="26" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="26" fillId="11" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="30" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="28" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="28" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="31" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="30" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="31" fillId="13" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="29" fillId="19" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="27" fillId="0" borderId="14" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="14" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="27" fillId="11" borderId="14" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="31" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="29" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="29" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="32" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="31" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="32" fillId="13" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2418,6 +2468,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="18.55" customHeight="1" s="109">
       <c r="A4" s="112" t="inlineStr">
         <is>
@@ -2808,6 +2859,7 @@
       <c r="A81" s="113" t="n"/>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="B0B1"/>
   <mergeCells count="7">
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="A28:B28"/>
@@ -2855,6 +2907,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="109">
       <c r="A3" s="123" t="inlineStr">
         <is>
@@ -3206,6 +3259,7 @@
         <v/>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="123" t="inlineStr">
         <is>
@@ -3499,14 +3553,15 @@
         </is>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
-      <c r="A41" s="117" t="inlineStr">
-        <is>
-          <t>Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com</t>
-        </is>
+      <c r="A41" s="117">
+        <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="B0B1"/>
   <autoFilter ref="A4:G22"/>
   <mergeCells count="1">
     <mergeCell ref="A39:E39"/>
@@ -3566,6 +3621,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1" s="109">
       <c r="A3" s="114" t="inlineStr">
         <is>
@@ -3573,6 +3629,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="123" t="inlineStr">
         <is>
@@ -3972,6 +4029,7 @@
         <v/>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="123" t="inlineStr">
         <is>
@@ -4071,6 +4129,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="136">
         <f>IF(Projects!$A$6="","",Projects!$A$6&amp;" — "&amp;Projects!$B$6)</f>
@@ -4365,6 +4424,7 @@
         <v/>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="136">
         <f>IF(Projects!$A$7="","",Projects!$A$7&amp;" — "&amp;Projects!$B$7)</f>
@@ -4659,6 +4719,7 @@
         <v/>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="136">
         <f>IF(Projects!$A$8="","",Projects!$A$8&amp;" — "&amp;Projects!$B$8)</f>
@@ -4953,6 +5014,7 @@
         <v/>
       </c>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="136">
         <f>IF(Projects!$A$9="","",Projects!$A$9&amp;" — "&amp;Projects!$B$9)</f>
@@ -5247,6 +5309,7 @@
         <v/>
       </c>
     </row>
+    <row r="38"/>
     <row r="39">
       <c r="A39" s="136">
         <f>IF(Projects!$A$10="","",Projects!$A$10&amp;" — "&amp;Projects!$B$10)</f>
@@ -5541,6 +5604,7 @@
         <v/>
       </c>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="136">
         <f>IF(Projects!$A$11="","",Projects!$A$11&amp;" — "&amp;Projects!$B$11)</f>
@@ -5835,6 +5899,7 @@
         <v/>
       </c>
     </row>
+    <row r="50"/>
     <row r="51">
       <c r="A51" s="136">
         <f>IF(Projects!$A$12="","",Projects!$A$12&amp;" — "&amp;Projects!$B$12)</f>
@@ -6129,6 +6194,7 @@
         <v/>
       </c>
     </row>
+    <row r="56"/>
     <row r="57">
       <c r="A57" s="136">
         <f>IF(Projects!$A$13="","",Projects!$A$13&amp;" — "&amp;Projects!$B$13)</f>
@@ -6423,6 +6489,8 @@
         <v/>
       </c>
     </row>
+    <row r="62"/>
+    <row r="63"/>
     <row r="64" ht="15" customHeight="1" s="109">
       <c r="A64" s="123" t="inlineStr">
         <is>
@@ -6692,14 +6760,15 @@
       <c r="G80" s="128" t="n"/>
       <c r="H80" s="128" t="n"/>
     </row>
+    <row r="81"/>
     <row r="82">
-      <c r="A82" s="117" t="inlineStr">
-        <is>
-          <t>Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com</t>
-        </is>
+      <c r="A82" s="117">
+        <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="B0B1"/>
   <mergeCells count="9">
     <mergeCell ref="A3:R3"/>
     <mergeCell ref="A21:R21"/>
@@ -6755,6 +6824,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1" s="109">
       <c r="A3" s="114" t="inlineStr">
         <is>
@@ -6762,6 +6832,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="123" t="inlineStr">
         <is>
@@ -6892,6 +6963,8 @@
         <v/>
       </c>
     </row>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="123" t="inlineStr">
         <is>
@@ -7844,14 +7917,15 @@
         <v>0.5</v>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
-      <c r="A40" s="117" t="inlineStr">
-        <is>
-          <t>Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com</t>
-        </is>
+      <c r="A40" s="117">
+        <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="B0B1"/>
   <mergeCells count="1">
     <mergeCell ref="A3:K3"/>
   </mergeCells>
@@ -7988,6 +8062,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="48" customHeight="1" s="109">
       <c r="A3" s="114" t="inlineStr">
         <is>
@@ -8500,6 +8575,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="123" t="inlineStr">
         <is>
@@ -8703,6 +8779,7 @@
         <v/>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="28" customHeight="1" s="109">
       <c r="A24" s="114" t="inlineStr">
         <is>
@@ -8710,14 +8787,15 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
-      <c r="A26" s="117" t="inlineStr">
-        <is>
-          <t>Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com</t>
-        </is>
+      <c r="A26" s="117">
+        <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="B0B1"/>
   <autoFilter ref="A4:P14"/>
   <mergeCells count="2">
     <mergeCell ref="A24:P24"/>
@@ -8802,6 +8880,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1" s="109">
       <c r="A3" s="114" t="inlineStr">
         <is>
@@ -8809,6 +8888,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="123" t="inlineStr">
         <is>
@@ -8823,6 +8903,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8" ht="24" customHeight="1" s="109">
       <c r="A8" s="137" t="inlineStr">
         <is>
@@ -8983,6 +9064,8 @@
       <c r="D23" s="217" t="n"/>
       <c r="E23" s="131" t="n"/>
     </row>
+    <row r="24"/>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="123" t="inlineStr">
         <is>
@@ -8997,6 +9080,7 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
@@ -9088,6 +9172,7 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="123" t="inlineStr">
         <is>
@@ -9102,6 +9187,7 @@
         </is>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
@@ -9179,6 +9265,7 @@
         <v/>
       </c>
     </row>
+    <row r="48"/>
     <row r="49">
       <c r="A49" s="123" t="inlineStr">
         <is>
@@ -9193,6 +9280,7 @@
         </is>
       </c>
     </row>
+    <row r="51"/>
     <row r="52" ht="24" customHeight="1" s="109">
       <c r="A52" s="137" t="inlineStr">
         <is>
@@ -9325,6 +9413,7 @@
         <v/>
       </c>
     </row>
+    <row r="58"/>
     <row r="59">
       <c r="A59" s="123" t="inlineStr">
         <is>
@@ -9339,6 +9428,7 @@
         </is>
       </c>
     </row>
+    <row r="61"/>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
@@ -9394,6 +9484,7 @@
         <v/>
       </c>
     </row>
+    <row r="67"/>
     <row r="68">
       <c r="A68" s="136">
         <f>"For "&amp;B30&amp;" from "&amp;TEXT(B35,"mm/dd/yyyy")&amp;" to "&amp;TEXT(B36,"mm/dd/yyyy")&amp;" ("&amp;B42&amp;" days): "&amp;TEXT(B66,"$#,##0")&amp;" fully burdened, ROM estimate."</f>
@@ -9407,14 +9498,15 @@
         </is>
       </c>
     </row>
+    <row r="70"/>
     <row r="71">
-      <c r="A71" s="117" t="inlineStr">
-        <is>
-          <t>Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com</t>
-        </is>
+      <c r="A71" s="117">
+        <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="B0B1"/>
   <mergeCells count="6">
     <mergeCell ref="A69:E69"/>
     <mergeCell ref="A50:E50"/>
@@ -9442,6 +9534,62 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" style="109" min="1" max="1"/>
+    <col width="34" customWidth="1" style="109" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="228" t="inlineStr">
+        <is>
+          <t>Acqlerate — License Record</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Licensed To (name or org):</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Email:</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>License Date:</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="229" t="inlineStr">
+        <is>
+          <t>This workbook is licensed for use by the individual or organization named above. Copyright Acqlerate. Redistribution, resale, or sharing outside that license without Acqlerate's written permission is prohibited.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -9472,6 +9620,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="123" t="inlineStr">
         <is>
@@ -9486,6 +9635,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="124" t="inlineStr">
         <is>
@@ -9546,6 +9696,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="123" t="inlineStr">
         <is>
@@ -9560,6 +9711,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="28" customHeight="1" s="109">
       <c r="A14" s="124" t="inlineStr">
         <is>
@@ -9590,6 +9742,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="117" t="inlineStr"/>
     </row>
@@ -9675,6 +9828,7 @@
         <v/>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="28" customHeight="1" s="109">
       <c r="A24" s="117" t="inlineStr">
         <is>
@@ -9682,6 +9836,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26" ht="42" customHeight="1" s="109">
       <c r="A26" s="114" t="inlineStr">
         <is>
@@ -9690,6 +9845,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="B0B1"/>
   <mergeCells count="10">
     <mergeCell ref="A24:F24"/>
     <mergeCell ref="C9:F9"/>
@@ -9744,6 +9900,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customFormat="1" customHeight="1" s="130">
       <c r="A3" s="114" t="inlineStr">
         <is>
@@ -9793,6 +9950,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="128" t="inlineStr">
         <is>
@@ -9937,6 +10095,7 @@
         <v/>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="133" t="n"/>
       <c r="B15" s="134" t="inlineStr">
@@ -9965,6 +10124,7 @@
         <v/>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="123" t="inlineStr">
         <is>
@@ -9979,6 +10139,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="136">
         <f>IF($A$6="","",$A$6&amp;" — "&amp;$B$6)</f>
@@ -10127,6 +10288,7 @@
         <v/>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="136">
         <f>IF($A$7="","",$A$7&amp;" — "&amp;$B$7)</f>
@@ -10275,6 +10437,7 @@
         <v/>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="136">
         <f>IF($A$8="","",$A$8&amp;" — "&amp;$B$8)</f>
@@ -10423,6 +10586,7 @@
         <v/>
       </c>
     </row>
+    <row r="43"/>
     <row r="44">
       <c r="A44" s="136">
         <f>IF($A$9="","",$A$9&amp;" — "&amp;$B$9)</f>
@@ -10571,6 +10735,7 @@
         <v/>
       </c>
     </row>
+    <row r="51"/>
     <row r="52">
       <c r="A52" s="136">
         <f>IF($A$10="","",$A$10&amp;" — "&amp;$B$10)</f>
@@ -10719,6 +10884,7 @@
         <v/>
       </c>
     </row>
+    <row r="59"/>
     <row r="60">
       <c r="A60" s="136">
         <f>IF($A$11="","",$A$11&amp;" — "&amp;$B$11)</f>
@@ -10867,6 +11033,7 @@
         <v/>
       </c>
     </row>
+    <row r="67"/>
     <row r="68">
       <c r="A68" s="136">
         <f>IF($A$12="","",$A$12&amp;" — "&amp;$B$12)</f>
@@ -11015,6 +11182,7 @@
         <v/>
       </c>
     </row>
+    <row r="75"/>
     <row r="76">
       <c r="A76" s="136">
         <f>IF($A$13="","",$A$13&amp;" — "&amp;$B$13)</f>
@@ -11163,14 +11331,16 @@
         <v/>
       </c>
     </row>
+    <row r="83"/>
+    <row r="84"/>
     <row r="85">
-      <c r="A85" s="117" t="inlineStr">
-        <is>
-          <t>Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com</t>
-        </is>
+      <c r="A85" s="117">
+        <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="B0B1"/>
   <autoFilter ref="A4:G13"/>
   <mergeCells count="9">
     <mergeCell ref="A36:G36"/>
@@ -11228,6 +11398,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="109">
       <c r="A3" s="118" t="inlineStr">
         <is>
@@ -11305,6 +11476,7 @@
         <v/>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="109">
       <c r="A11" s="148" t="inlineStr">
         <is>
@@ -11389,6 +11561,7 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="33.75" customHeight="1" s="109">
       <c r="A20" s="151" t="inlineStr">
         <is>
@@ -12418,14 +12591,15 @@
         <v/>
       </c>
     </row>
+    <row r="33"/>
     <row r="34" ht="15" customHeight="1" s="109">
-      <c r="A34" s="111" t="inlineStr">
-        <is>
-          <t>Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com</t>
-        </is>
+      <c r="A34" s="120">
+        <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="B0B1"/>
   <mergeCells count="15">
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A3:B3"/>
@@ -13138,13 +13312,13 @@
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="109">
-      <c r="A21" s="111" t="inlineStr">
-        <is>
-          <t>Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com</t>
-        </is>
+      <c r="A21" s="120">
+        <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="B0B1"/>
   <mergeCells count="1">
     <mergeCell ref="A20:N20"/>
   </mergeCells>
@@ -13217,6 +13391,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1" s="109">
       <c r="A3" s="114" t="inlineStr">
         <is>
@@ -14060,14 +14235,15 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
-      <c r="A22" s="117" t="inlineStr">
-        <is>
-          <t>Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com</t>
-        </is>
+      <c r="A22" s="117">
+        <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="B0B1"/>
   <mergeCells count="18">
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="P4:Q4"/>
@@ -14176,6 +14352,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="109">
       <c r="A3" s="117" t="inlineStr">
         <is>
@@ -17652,6 +17829,7 @@
         <v/>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="123" t="inlineStr">
         <is>
@@ -18211,6 +18389,7 @@
         <v/>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" s="117" t="inlineStr">
         <is>
@@ -18218,14 +18397,15 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
     <row r="44">
-      <c r="A44" s="117" t="inlineStr">
-        <is>
-          <t>Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com</t>
-        </is>
+      <c r="A44" s="117">
+        <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="B0B1"/>
   <autoFilter ref="A4:G25"/>
   <mergeCells count="23">
     <mergeCell ref="C4:C5"/>
@@ -18377,6 +18557,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="109">
       <c r="A3" s="123" t="inlineStr">
         <is>
@@ -18728,6 +18909,7 @@
         <v/>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="123" t="inlineStr">
         <is>
@@ -19021,14 +19203,15 @@
         </is>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
-      <c r="A41" s="117" t="inlineStr">
-        <is>
-          <t>Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com</t>
-        </is>
+      <c r="A41" s="117">
+        <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="B0B1"/>
   <autoFilter ref="A4:G22"/>
   <mergeCells count="1">
     <mergeCell ref="A39:E39"/>
@@ -19077,6 +19260,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="109">
       <c r="A3" s="123" t="inlineStr">
         <is>
@@ -19428,6 +19612,7 @@
         <v/>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="123" t="inlineStr">
         <is>
@@ -19721,14 +19906,15 @@
         </is>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
-      <c r="A41" s="117" t="inlineStr">
-        <is>
-          <t>Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com</t>
-        </is>
+      <c r="A41" s="117">
+        <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="B0B1"/>
   <autoFilter ref="A4:G22"/>
   <mergeCells count="1">
     <mergeCell ref="A39:E39"/>

</xml_diff>

<commit_message>
Fix G&A methodology: apply G&A to subcontractor M&S-burdened cost
Sub Travel/ODC/M&E cost draws M&S markup, and G&A is then charged on
top of that M&S-burdened sub cost (same as it's charged on Prime
cost) — not excluded from G&A as the prior formulas assumed. Fixes
both the cost tracker engine and the distributed Excel template
(Dashboard G&A/Fee formulas + Rates tab tooltips), verified against
an independent recalculation.

Also sends users from the tracker intro straight into Task Orders
(not Projects) per the intended setup flow, and auto-opens a newly
created Task Order so adding its first project is one click away.
</commit_message>
<xml_diff>
--- a/client/public/examples/cost-and-burn-rate-tracker.xlsx
+++ b/client/public/examples/cost-and-burn-rate-tracker.xlsx
@@ -37,7 +37,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="166" formatCode="\$#,##0"/>
@@ -45,9 +45,8 @@
     <numFmt numFmtId="168" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="169" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
-    <numFmt numFmtId="171" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="171" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="172" formatCode="m/d/yyyy"/>
-    <numFmt numFmtId="173" formatCode="0.00&quot;x&quot;"/>
   </numFmts>
   <fonts count="36">
     <font>
@@ -395,7 +394,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -570,6 +569,55 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -581,7 +629,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="230">
+  <cellXfs count="235">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1076,7 +1124,7 @@
     <xf numFmtId="169" fontId="31" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="173" fontId="29" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="29" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="170" fontId="10" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1112,7 +1160,7 @@
     <xf numFmtId="169" fontId="31" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="173" fontId="29" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="29" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="170" fontId="10" fillId="6" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1192,6 +1240,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="171" fontId="29" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="171" fontId="29" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1741,26 +1798,9 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="1.2"/>
-          <min val="0"/>
         </scaling>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>% of CLIN Funding Used</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0%" sourceLinked="0"/>
+        <majorGridlines/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -1844,6 +1884,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1874,6 +1917,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1926,6 +1972,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1956,6 +2005,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1986,6 +2038,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2016,6 +2071,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2046,6 +2104,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2168,6 +2229,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2198,6 +2262,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2228,6 +2295,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2258,6 +2328,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2468,7 +2541,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="18.55" customHeight="1" s="109">
       <c r="A4" s="112" t="inlineStr">
         <is>
@@ -2907,7 +2979,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="109">
       <c r="A3" s="123" t="inlineStr">
         <is>
@@ -3259,7 +3330,6 @@
         <v/>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="123" t="inlineStr">
         <is>
@@ -3553,7 +3623,6 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="117">
         <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
@@ -3621,7 +3690,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="28" customHeight="1" s="109">
       <c r="A3" s="114" t="inlineStr">
         <is>
@@ -3629,7 +3697,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="123" t="inlineStr">
         <is>
@@ -4029,7 +4096,6 @@
         <v/>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="123" t="inlineStr">
         <is>
@@ -4129,7 +4195,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="136">
         <f>IF(Projects!$A$6="","",Projects!$A$6&amp;" — "&amp;Projects!$B$6)</f>
@@ -4424,7 +4489,6 @@
         <v/>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="136">
         <f>IF(Projects!$A$7="","",Projects!$A$7&amp;" — "&amp;Projects!$B$7)</f>
@@ -4719,7 +4783,6 @@
         <v/>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="136">
         <f>IF(Projects!$A$8="","",Projects!$A$8&amp;" — "&amp;Projects!$B$8)</f>
@@ -5014,7 +5077,6 @@
         <v/>
       </c>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="136">
         <f>IF(Projects!$A$9="","",Projects!$A$9&amp;" — "&amp;Projects!$B$9)</f>
@@ -5309,7 +5371,6 @@
         <v/>
       </c>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="A39" s="136">
         <f>IF(Projects!$A$10="","",Projects!$A$10&amp;" — "&amp;Projects!$B$10)</f>
@@ -5604,7 +5665,6 @@
         <v/>
       </c>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="A45" s="136">
         <f>IF(Projects!$A$11="","",Projects!$A$11&amp;" — "&amp;Projects!$B$11)</f>
@@ -5899,7 +5959,6 @@
         <v/>
       </c>
     </row>
-    <row r="50"/>
     <row r="51">
       <c r="A51" s="136">
         <f>IF(Projects!$A$12="","",Projects!$A$12&amp;" — "&amp;Projects!$B$12)</f>
@@ -6194,7 +6253,6 @@
         <v/>
       </c>
     </row>
-    <row r="56"/>
     <row r="57">
       <c r="A57" s="136">
         <f>IF(Projects!$A$13="","",Projects!$A$13&amp;" — "&amp;Projects!$B$13)</f>
@@ -6489,8 +6547,6 @@
         <v/>
       </c>
     </row>
-    <row r="62"/>
-    <row r="63"/>
     <row r="64" ht="15" customHeight="1" s="109">
       <c r="A64" s="123" t="inlineStr">
         <is>
@@ -6760,7 +6816,6 @@
       <c r="G80" s="128" t="n"/>
       <c r="H80" s="128" t="n"/>
     </row>
-    <row r="81"/>
     <row r="82">
       <c r="A82" s="117">
         <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
@@ -6824,7 +6879,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="28" customHeight="1" s="109">
       <c r="A3" s="114" t="inlineStr">
         <is>
@@ -6832,7 +6886,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="123" t="inlineStr">
         <is>
@@ -6963,8 +7016,6 @@
         <v/>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="123" t="inlineStr">
         <is>
@@ -7917,7 +7968,6 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="117">
         <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
@@ -8062,7 +8112,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="48" customHeight="1" s="109">
       <c r="A3" s="114" t="inlineStr">
         <is>
@@ -8575,7 +8624,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="123" t="inlineStr">
         <is>
@@ -8779,7 +8827,6 @@
         <v/>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="28" customHeight="1" s="109">
       <c r="A24" s="114" t="inlineStr">
         <is>
@@ -8787,7 +8834,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="117">
         <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
@@ -8880,7 +8926,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="30" customHeight="1" s="109">
       <c r="A3" s="114" t="inlineStr">
         <is>
@@ -8888,7 +8933,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="123" t="inlineStr">
         <is>
@@ -8903,7 +8947,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="24" customHeight="1" s="109">
       <c r="A8" s="137" t="inlineStr">
         <is>
@@ -9064,8 +9107,6 @@
       <c r="D23" s="217" t="n"/>
       <c r="E23" s="131" t="n"/>
     </row>
-    <row r="24"/>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="123" t="inlineStr">
         <is>
@@ -9080,9 +9121,8 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="108" t="inlineStr">
         <is>
           <t>Duty Location</t>
         </is>
@@ -9095,7 +9135,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="108" t="inlineStr">
         <is>
           <t>Role / LCAT</t>
         </is>
@@ -9107,7 +9147,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="108" t="inlineStr">
         <is>
           <t>Employee Type</t>
         </is>
@@ -9119,7 +9159,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="108" t="inlineStr">
         <is>
           <t>Annual Salary (Exempt only)</t>
         </is>
@@ -9129,7 +9169,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="108" t="inlineStr">
         <is>
           <t>Direct Hourly Rate (Non-Exempt only)</t>
         </is>
@@ -9137,7 +9177,7 @@
       <c r="B33" s="218" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="108" t="inlineStr">
         <is>
           <t>Standard Annual Hours</t>
         </is>
@@ -9147,7 +9187,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="108" t="inlineStr">
         <is>
           <t>Start Date</t>
         </is>
@@ -9157,7 +9197,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="108" t="inlineStr">
         <is>
           <t>End Date</t>
         </is>
@@ -9172,7 +9212,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="123" t="inlineStr">
         <is>
@@ -9187,9 +9226,8 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="108" t="inlineStr">
         <is>
           <t>Straight-Time Rate $/hr</t>
         </is>
@@ -9200,7 +9238,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="108" t="inlineStr">
         <is>
           <t>Days in Period</t>
         </is>
@@ -9211,7 +9249,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="108" t="inlineStr">
         <is>
           <t>Estimated Hours in Period</t>
         </is>
@@ -9222,7 +9260,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="108" t="inlineStr">
         <is>
           <t>Direct Labor $</t>
         </is>
@@ -9233,7 +9271,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="108" t="inlineStr">
         <is>
           <t>Fringe $</t>
         </is>
@@ -9244,7 +9282,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="108" t="inlineStr">
         <is>
           <t>OH $</t>
         </is>
@@ -9265,7 +9303,6 @@
         <v/>
       </c>
     </row>
-    <row r="48"/>
     <row r="49">
       <c r="A49" s="123" t="inlineStr">
         <is>
@@ -9280,7 +9317,6 @@
         </is>
       </c>
     </row>
-    <row r="51"/>
     <row r="52" ht="24" customHeight="1" s="109">
       <c r="A52" s="137" t="inlineStr">
         <is>
@@ -9413,7 +9449,6 @@
         <v/>
       </c>
     </row>
-    <row r="58"/>
     <row r="59">
       <c r="A59" s="123" t="inlineStr">
         <is>
@@ -9428,9 +9463,8 @@
         </is>
       </c>
     </row>
-    <row r="61"/>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="108" t="inlineStr">
         <is>
           <t>Subtotal (Labor + Adders) $</t>
         </is>
@@ -9441,7 +9475,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="108" t="inlineStr">
         <is>
           <t>G&amp;A $</t>
         </is>
@@ -9452,7 +9486,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="108" t="inlineStr">
         <is>
           <t>Total Cost $</t>
         </is>
@@ -9463,7 +9497,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="108" t="inlineStr">
         <is>
           <t>Fee $</t>
         </is>
@@ -9484,7 +9518,6 @@
         <v/>
       </c>
     </row>
-    <row r="67"/>
     <row r="68">
       <c r="A68" s="136">
         <f>"For "&amp;B30&amp;" from "&amp;TEXT(B35,"mm/dd/yyyy")&amp;" to "&amp;TEXT(B36,"mm/dd/yyyy")&amp;" ("&amp;B42&amp;" days): "&amp;TEXT(B66,"$#,##0")&amp;" fully burdened, ROM estimate."</f>
@@ -9498,7 +9531,6 @@
         </is>
       </c>
     </row>
-    <row r="70"/>
     <row r="71">
       <c r="A71" s="117">
         <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
@@ -9555,28 +9587,28 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="108" t="inlineStr">
         <is>
           <t>Licensed To (name or org):</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" s="108" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="108" t="inlineStr">
         <is>
           <t>Email:</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" s="108" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="108" t="inlineStr">
         <is>
           <t>License Date:</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" s="108" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="229" t="inlineStr">
@@ -9620,7 +9652,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="123" t="inlineStr">
         <is>
@@ -9635,7 +9666,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="124" t="inlineStr">
         <is>
@@ -9677,7 +9707,7 @@
       </c>
       <c r="C8" s="114" t="inlineStr">
         <is>
-          <t>Applied to PRIME-sourced cost only: Prime fully burdened labor + Prime-bought Travel/ODC/M&amp;E. Covers company-wide G&amp;A: executive, finance, HR, business development.</t>
+          <t>Applied to Prime-sourced cost (fully burdened labor + Prime-bought Travel/ODC/M&amp;E) AND to Sub-sourced Travel/ODC/M&amp;E after the M&amp;S markup (below) is added to it. Covers company-wide G&amp;A: executive, finance, HR, business development.</t>
         </is>
       </c>
     </row>
@@ -9692,11 +9722,10 @@
       </c>
       <c r="C9" s="114" t="inlineStr">
         <is>
-          <t>Applied to SUB-sourced Travel/ODC/M&amp;E only — not Sub labor, which passes through at raw cost. Your Sub already carries their own G&amp;A in what they bill you, so this is a smaller subcontract administration/handling markup, not a second G&amp;A.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
+          <t>Applied to SUB-sourced Travel/ODC/M&amp;E only — not Sub labor, which passes through at raw cost. This is a subcontract administration/handling markup. G&amp;A (above) is then charged on top of Sub cost plus this M&amp;S markup, the same way it's charged on Prime cost.</t>
+        </is>
+      </c>
+    </row>
     <row r="11">
       <c r="A11" s="123" t="inlineStr">
         <is>
@@ -9711,7 +9740,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="28" customHeight="1" s="109">
       <c r="A14" s="124" t="inlineStr">
         <is>
@@ -9742,7 +9770,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="117" t="inlineStr"/>
     </row>
@@ -9828,7 +9855,6 @@
         <v/>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="28" customHeight="1" s="109">
       <c r="A24" s="117" t="inlineStr">
         <is>
@@ -9836,7 +9862,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26" ht="42" customHeight="1" s="109">
       <c r="A26" s="114" t="inlineStr">
         <is>
@@ -9900,7 +9925,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="30" customFormat="1" customHeight="1" s="130">
       <c r="A3" s="114" t="inlineStr">
         <is>
@@ -9950,7 +9974,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="128" t="inlineStr">
         <is>
@@ -10095,7 +10118,6 @@
         <v/>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="133" t="n"/>
       <c r="B15" s="134" t="inlineStr">
@@ -10124,7 +10146,6 @@
         <v/>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="123" t="inlineStr">
         <is>
@@ -10139,7 +10160,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="136">
         <f>IF($A$6="","",$A$6&amp;" — "&amp;$B$6)</f>
@@ -10288,7 +10308,6 @@
         <v/>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="136">
         <f>IF($A$7="","",$A$7&amp;" — "&amp;$B$7)</f>
@@ -10437,7 +10456,6 @@
         <v/>
       </c>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="136">
         <f>IF($A$8="","",$A$8&amp;" — "&amp;$B$8)</f>
@@ -10586,7 +10604,6 @@
         <v/>
       </c>
     </row>
-    <row r="43"/>
     <row r="44">
       <c r="A44" s="136">
         <f>IF($A$9="","",$A$9&amp;" — "&amp;$B$9)</f>
@@ -10735,7 +10752,6 @@
         <v/>
       </c>
     </row>
-    <row r="51"/>
     <row r="52">
       <c r="A52" s="136">
         <f>IF($A$10="","",$A$10&amp;" — "&amp;$B$10)</f>
@@ -10884,7 +10900,6 @@
         <v/>
       </c>
     </row>
-    <row r="59"/>
     <row r="60">
       <c r="A60" s="136">
         <f>IF($A$11="","",$A$11&amp;" — "&amp;$B$11)</f>
@@ -11033,7 +11048,6 @@
         <v/>
       </c>
     </row>
-    <row r="67"/>
     <row r="68">
       <c r="A68" s="136">
         <f>IF($A$12="","",$A$12&amp;" — "&amp;$B$12)</f>
@@ -11182,7 +11196,6 @@
         <v/>
       </c>
     </row>
-    <row r="75"/>
     <row r="76">
       <c r="A76" s="136">
         <f>IF($A$13="","",$A$13&amp;" — "&amp;$B$13)</f>
@@ -11331,8 +11344,6 @@
         <v/>
       </c>
     </row>
-    <row r="83"/>
-    <row r="84"/>
     <row r="85">
       <c r="A85" s="117">
         <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
@@ -11398,7 +11409,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="109">
       <c r="A3" s="118" t="inlineStr">
         <is>
@@ -11476,7 +11486,6 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="109">
       <c r="A11" s="148" t="inlineStr">
         <is>
@@ -11561,7 +11570,6 @@
         <v/>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="33.75" customHeight="1" s="109">
       <c r="A20" s="151" t="inlineStr">
         <is>
@@ -11700,7 +11708,7 @@
         <v/>
       </c>
       <c r="I21" s="155">
-        <f>IF(H21="","",Q21*Rates!$B$8)</f>
+        <f>IF(H21="","",(Q21+R21+S21)*Rates!$B$8)</f>
         <v/>
       </c>
       <c r="J21" s="154">
@@ -11708,7 +11716,7 @@
         <v/>
       </c>
       <c r="K21" s="155">
-        <f>IF(H21="","",(Labor!F29+IFERROR(Labor!F29/Q21*I21,0)+Labor!G29)*Rates!$C$19+(Travel!D27+IFERROR(Travel!D27/Q21*I21,0)+Travel!E27+IFERROR(Travel!E27/R21*S21,0))*Rates!$C$20+(ODCs!D27+IFERROR(ODCs!D27/Q21*I21,0)+ODCs!E27+IFERROR(ODCs!E27/R21*S21,0))*Rates!$C$21+('M&amp;E'!D27+IFERROR('M&amp;E'!D27/Q21*I21,0)+'M&amp;E'!E27+IFERROR('M&amp;E'!E27/R21*S21,0))*Rates!$C$22)</f>
+        <f>IF(H21="","",(Labor!F29+IFERROR(Labor!F29/(Q21+R21+S21)*I21,0)+Labor!G29)*Rates!$C$19+(Travel!D27+IFERROR(Travel!D27/(Q21+R21+S21)*I21,0)+Travel!E27+IFERROR(Travel!E27/R21*S21,0)+IFERROR((Travel!E27+Travel!E27/R21*S21)/(Q21+R21+S21)*I21,0))*Rates!$C$20+(ODCs!D27+IFERROR(ODCs!D27/(Q21+R21+S21)*I21,0)+ODCs!E27+IFERROR(ODCs!E27/R21*S21,0)+IFERROR((ODCs!E27+ODCs!E27/R21*S21)/(Q21+R21+S21)*I21,0))*Rates!$C$21+('M&amp;E'!D27+IFERROR('M&amp;E'!D27/(Q21+R21+S21)*I21,0)+'M&amp;E'!E27+IFERROR('M&amp;E'!E27/R21*S21,0)+IFERROR(('M&amp;E'!E27+'M&amp;E'!E27/R21*S21)/(Q21+R21+S21)*I21,0))*Rates!$C$22)</f>
         <v/>
       </c>
       <c r="L21" s="154">
@@ -11777,7 +11785,7 @@
         <v/>
       </c>
       <c r="I22" s="162">
-        <f>IF(H22="","",Q22*Rates!$B$8)</f>
+        <f>IF(H22="","",(Q22+R22+S22)*Rates!$B$8)</f>
         <v/>
       </c>
       <c r="J22" s="161">
@@ -11785,7 +11793,7 @@
         <v/>
       </c>
       <c r="K22" s="162">
-        <f>IF(H22="","",(Labor!F30+IFERROR(Labor!F30/Q22*I22,0)+Labor!G30)*Rates!$C$19+(Travel!D28+IFERROR(Travel!D28/Q22*I22,0)+Travel!E28+IFERROR(Travel!E28/R22*S22,0))*Rates!$C$20+(ODCs!D28+IFERROR(ODCs!D28/Q22*I22,0)+ODCs!E28+IFERROR(ODCs!E28/R22*S22,0))*Rates!$C$21+('M&amp;E'!D28+IFERROR('M&amp;E'!D28/Q22*I22,0)+'M&amp;E'!E28+IFERROR('M&amp;E'!E28/R22*S22,0))*Rates!$C$22)</f>
+        <f>IF(H22="","",(Labor!F30+IFERROR(Labor!F30/(Q22+R22+S22)*I22,0)+Labor!G30)*Rates!$C$19+(Travel!D28+IFERROR(Travel!D28/(Q22+R22+S22)*I22,0)+Travel!E28+IFERROR(Travel!E28/R22*S22,0)+IFERROR((Travel!E28+Travel!E28/R22*S22)/(Q22+R22+S22)*I22,0))*Rates!$C$20+(ODCs!D28+IFERROR(ODCs!D28/(Q22+R22+S22)*I22,0)+ODCs!E28+IFERROR(ODCs!E28/R22*S22,0)+IFERROR((ODCs!E28+ODCs!E28/R22*S22)/(Q22+R22+S22)*I22,0))*Rates!$C$21+('M&amp;E'!D28+IFERROR('M&amp;E'!D28/(Q22+R22+S22)*I22,0)+'M&amp;E'!E28+IFERROR('M&amp;E'!E28/R22*S22,0)+IFERROR(('M&amp;E'!E28+'M&amp;E'!E28/R22*S22)/(Q22+R22+S22)*I22,0))*Rates!$C$22)</f>
         <v/>
       </c>
       <c r="L22" s="161">
@@ -11854,7 +11862,7 @@
         <v/>
       </c>
       <c r="I23" s="155">
-        <f>IF(H23="","",Q23*Rates!$B$8)</f>
+        <f>IF(H23="","",(Q23+R23+S23)*Rates!$B$8)</f>
         <v/>
       </c>
       <c r="J23" s="154">
@@ -11862,7 +11870,7 @@
         <v/>
       </c>
       <c r="K23" s="155">
-        <f>IF(H23="","",(Labor!F31+IFERROR(Labor!F31/Q23*I23,0)+Labor!G31)*Rates!$C$19+(Travel!D29+IFERROR(Travel!D29/Q23*I23,0)+Travel!E29+IFERROR(Travel!E29/R23*S23,0))*Rates!$C$20+(ODCs!D29+IFERROR(ODCs!D29/Q23*I23,0)+ODCs!E29+IFERROR(ODCs!E29/R23*S23,0))*Rates!$C$21+('M&amp;E'!D29+IFERROR('M&amp;E'!D29/Q23*I23,0)+'M&amp;E'!E29+IFERROR('M&amp;E'!E29/R23*S23,0))*Rates!$C$22)</f>
+        <f>IF(H23="","",(Labor!F31+IFERROR(Labor!F31/(Q23+R23+S23)*I23,0)+Labor!G31)*Rates!$C$19+(Travel!D29+IFERROR(Travel!D29/(Q23+R23+S23)*I23,0)+Travel!E29+IFERROR(Travel!E29/R23*S23,0)+IFERROR((Travel!E29+Travel!E29/R23*S23)/(Q23+R23+S23)*I23,0))*Rates!$C$20+(ODCs!D29+IFERROR(ODCs!D29/(Q23+R23+S23)*I23,0)+ODCs!E29+IFERROR(ODCs!E29/R23*S23,0)+IFERROR((ODCs!E29+ODCs!E29/R23*S23)/(Q23+R23+S23)*I23,0))*Rates!$C$21+('M&amp;E'!D29+IFERROR('M&amp;E'!D29/(Q23+R23+S23)*I23,0)+'M&amp;E'!E29+IFERROR('M&amp;E'!E29/R23*S23,0)+IFERROR(('M&amp;E'!E29+'M&amp;E'!E29/R23*S23)/(Q23+R23+S23)*I23,0))*Rates!$C$22)</f>
         <v/>
       </c>
       <c r="L23" s="154">
@@ -11931,7 +11939,7 @@
         <v/>
       </c>
       <c r="I24" s="162">
-        <f>IF(H24="","",Q24*Rates!$B$8)</f>
+        <f>IF(H24="","",(Q24+R24+S24)*Rates!$B$8)</f>
         <v/>
       </c>
       <c r="J24" s="161">
@@ -11939,7 +11947,7 @@
         <v/>
       </c>
       <c r="K24" s="162">
-        <f>IF(H24="","",(Labor!F32+IFERROR(Labor!F32/Q24*I24,0)+Labor!G32)*Rates!$C$19+(Travel!D30+IFERROR(Travel!D30/Q24*I24,0)+Travel!E30+IFERROR(Travel!E30/R24*S24,0))*Rates!$C$20+(ODCs!D30+IFERROR(ODCs!D30/Q24*I24,0)+ODCs!E30+IFERROR(ODCs!E30/R24*S24,0))*Rates!$C$21+('M&amp;E'!D30+IFERROR('M&amp;E'!D30/Q24*I24,0)+'M&amp;E'!E30+IFERROR('M&amp;E'!E30/R24*S24,0))*Rates!$C$22)</f>
+        <f>IF(H24="","",(Labor!F32+IFERROR(Labor!F32/(Q24+R24+S24)*I24,0)+Labor!G32)*Rates!$C$19+(Travel!D30+IFERROR(Travel!D30/(Q24+R24+S24)*I24,0)+Travel!E30+IFERROR(Travel!E30/R24*S24,0)+IFERROR((Travel!E30+Travel!E30/R24*S24)/(Q24+R24+S24)*I24,0))*Rates!$C$20+(ODCs!D30+IFERROR(ODCs!D30/(Q24+R24+S24)*I24,0)+ODCs!E30+IFERROR(ODCs!E30/R24*S24,0)+IFERROR((ODCs!E30+ODCs!E30/R24*S24)/(Q24+R24+S24)*I24,0))*Rates!$C$21+('M&amp;E'!D30+IFERROR('M&amp;E'!D30/(Q24+R24+S24)*I24,0)+'M&amp;E'!E30+IFERROR('M&amp;E'!E30/R24*S24,0)+IFERROR(('M&amp;E'!E30+'M&amp;E'!E30/R24*S24)/(Q24+R24+S24)*I24,0))*Rates!$C$22)</f>
         <v/>
       </c>
       <c r="L24" s="161">
@@ -12008,7 +12016,7 @@
         <v/>
       </c>
       <c r="I25" s="155">
-        <f>IF(H25="","",Q25*Rates!$B$8)</f>
+        <f>IF(H25="","",(Q25+R25+S25)*Rates!$B$8)</f>
         <v/>
       </c>
       <c r="J25" s="154">
@@ -12016,7 +12024,7 @@
         <v/>
       </c>
       <c r="K25" s="155">
-        <f>IF(H25="","",(Labor!F33+IFERROR(Labor!F33/Q25*I25,0)+Labor!G33)*Rates!$C$19+(Travel!D31+IFERROR(Travel!D31/Q25*I25,0)+Travel!E31+IFERROR(Travel!E31/R25*S25,0))*Rates!$C$20+(ODCs!D31+IFERROR(ODCs!D31/Q25*I25,0)+ODCs!E31+IFERROR(ODCs!E31/R25*S25,0))*Rates!$C$21+('M&amp;E'!D31+IFERROR('M&amp;E'!D31/Q25*I25,0)+'M&amp;E'!E31+IFERROR('M&amp;E'!E31/R25*S25,0))*Rates!$C$22)</f>
+        <f>IF(H25="","",(Labor!F33+IFERROR(Labor!F33/(Q25+R25+S25)*I25,0)+Labor!G33)*Rates!$C$19+(Travel!D31+IFERROR(Travel!D31/(Q25+R25+S25)*I25,0)+Travel!E31+IFERROR(Travel!E31/R25*S25,0)+IFERROR((Travel!E31+Travel!E31/R25*S25)/(Q25+R25+S25)*I25,0))*Rates!$C$20+(ODCs!D31+IFERROR(ODCs!D31/(Q25+R25+S25)*I25,0)+ODCs!E31+IFERROR(ODCs!E31/R25*S25,0)+IFERROR((ODCs!E31+ODCs!E31/R25*S25)/(Q25+R25+S25)*I25,0))*Rates!$C$21+('M&amp;E'!D31+IFERROR('M&amp;E'!D31/(Q25+R25+S25)*I25,0)+'M&amp;E'!E31+IFERROR('M&amp;E'!E31/R25*S25,0)+IFERROR(('M&amp;E'!E31+'M&amp;E'!E31/R25*S25)/(Q25+R25+S25)*I25,0))*Rates!$C$22)</f>
         <v/>
       </c>
       <c r="L25" s="154">
@@ -12085,7 +12093,7 @@
         <v/>
       </c>
       <c r="I26" s="162">
-        <f>IF(H26="","",Q26*Rates!$B$8)</f>
+        <f>IF(H26="","",(Q26+R26+S26)*Rates!$B$8)</f>
         <v/>
       </c>
       <c r="J26" s="161">
@@ -12093,7 +12101,7 @@
         <v/>
       </c>
       <c r="K26" s="162">
-        <f>IF(H26="","",(Labor!F34+IFERROR(Labor!F34/Q26*I26,0)+Labor!G34)*Rates!$C$19+(Travel!D32+IFERROR(Travel!D32/Q26*I26,0)+Travel!E32+IFERROR(Travel!E32/R26*S26,0))*Rates!$C$20+(ODCs!D32+IFERROR(ODCs!D32/Q26*I26,0)+ODCs!E32+IFERROR(ODCs!E32/R26*S26,0))*Rates!$C$21+('M&amp;E'!D32+IFERROR('M&amp;E'!D32/Q26*I26,0)+'M&amp;E'!E32+IFERROR('M&amp;E'!E32/R26*S26,0))*Rates!$C$22)</f>
+        <f>IF(H26="","",(Labor!F34+IFERROR(Labor!F34/(Q26+R26+S26)*I26,0)+Labor!G34)*Rates!$C$19+(Travel!D32+IFERROR(Travel!D32/(Q26+R26+S26)*I26,0)+Travel!E32+IFERROR(Travel!E32/R26*S26,0)+IFERROR((Travel!E32+Travel!E32/R26*S26)/(Q26+R26+S26)*I26,0))*Rates!$C$20+(ODCs!D32+IFERROR(ODCs!D32/(Q26+R26+S26)*I26,0)+ODCs!E32+IFERROR(ODCs!E32/R26*S26,0)+IFERROR((ODCs!E32+ODCs!E32/R26*S26)/(Q26+R26+S26)*I26,0))*Rates!$C$21+('M&amp;E'!D32+IFERROR('M&amp;E'!D32/(Q26+R26+S26)*I26,0)+'M&amp;E'!E32+IFERROR('M&amp;E'!E32/R26*S26,0)+IFERROR(('M&amp;E'!E32+'M&amp;E'!E32/R26*S26)/(Q26+R26+S26)*I26,0))*Rates!$C$22)</f>
         <v/>
       </c>
       <c r="L26" s="161">
@@ -12162,7 +12170,7 @@
         <v/>
       </c>
       <c r="I27" s="155">
-        <f>IF(H27="","",Q27*Rates!$B$8)</f>
+        <f>IF(H27="","",(Q27+R27+S27)*Rates!$B$8)</f>
         <v/>
       </c>
       <c r="J27" s="154">
@@ -12170,7 +12178,7 @@
         <v/>
       </c>
       <c r="K27" s="155">
-        <f>IF(H27="","",(Labor!F35+IFERROR(Labor!F35/Q27*I27,0)+Labor!G35)*Rates!$C$19+(Travel!D33+IFERROR(Travel!D33/Q27*I27,0)+Travel!E33+IFERROR(Travel!E33/R27*S27,0))*Rates!$C$20+(ODCs!D33+IFERROR(ODCs!D33/Q27*I27,0)+ODCs!E33+IFERROR(ODCs!E33/R27*S27,0))*Rates!$C$21+('M&amp;E'!D33+IFERROR('M&amp;E'!D33/Q27*I27,0)+'M&amp;E'!E33+IFERROR('M&amp;E'!E33/R27*S27,0))*Rates!$C$22)</f>
+        <f>IF(H27="","",(Labor!F35+IFERROR(Labor!F35/(Q27+R27+S27)*I27,0)+Labor!G35)*Rates!$C$19+(Travel!D33+IFERROR(Travel!D33/(Q27+R27+S27)*I27,0)+Travel!E33+IFERROR(Travel!E33/R27*S27,0)+IFERROR((Travel!E33+Travel!E33/R27*S27)/(Q27+R27+S27)*I27,0))*Rates!$C$20+(ODCs!D33+IFERROR(ODCs!D33/(Q27+R27+S27)*I27,0)+ODCs!E33+IFERROR(ODCs!E33/R27*S27,0)+IFERROR((ODCs!E33+ODCs!E33/R27*S27)/(Q27+R27+S27)*I27,0))*Rates!$C$21+('M&amp;E'!D33+IFERROR('M&amp;E'!D33/(Q27+R27+S27)*I27,0)+'M&amp;E'!E33+IFERROR('M&amp;E'!E33/R27*S27,0)+IFERROR(('M&amp;E'!E33+'M&amp;E'!E33/R27*S27)/(Q27+R27+S27)*I27,0))*Rates!$C$22)</f>
         <v/>
       </c>
       <c r="L27" s="154">
@@ -12239,7 +12247,7 @@
         <v/>
       </c>
       <c r="I28" s="162">
-        <f>IF(H28="","",Q28*Rates!$B$8)</f>
+        <f>IF(H28="","",(Q28+R28+S28)*Rates!$B$8)</f>
         <v/>
       </c>
       <c r="J28" s="161">
@@ -12247,7 +12255,7 @@
         <v/>
       </c>
       <c r="K28" s="162">
-        <f>IF(H28="","",(Labor!F36+IFERROR(Labor!F36/Q28*I28,0)+Labor!G36)*Rates!$C$19+(Travel!D34+IFERROR(Travel!D34/Q28*I28,0)+Travel!E34+IFERROR(Travel!E34/R28*S28,0))*Rates!$C$20+(ODCs!D34+IFERROR(ODCs!D34/Q28*I28,0)+ODCs!E34+IFERROR(ODCs!E34/R28*S28,0))*Rates!$C$21+('M&amp;E'!D34+IFERROR('M&amp;E'!D34/Q28*I28,0)+'M&amp;E'!E34+IFERROR('M&amp;E'!E34/R28*S28,0))*Rates!$C$22)</f>
+        <f>IF(H28="","",(Labor!F36+IFERROR(Labor!F36/(Q28+R28+S28)*I28,0)+Labor!G36)*Rates!$C$19+(Travel!D34+IFERROR(Travel!D34/(Q28+R28+S28)*I28,0)+Travel!E34+IFERROR(Travel!E34/R28*S28,0)+IFERROR((Travel!E34+Travel!E34/R28*S28)/(Q28+R28+S28)*I28,0))*Rates!$C$20+(ODCs!D34+IFERROR(ODCs!D34/(Q28+R28+S28)*I28,0)+ODCs!E34+IFERROR(ODCs!E34/R28*S28,0)+IFERROR((ODCs!E34+ODCs!E34/R28*S28)/(Q28+R28+S28)*I28,0))*Rates!$C$21+('M&amp;E'!D34+IFERROR('M&amp;E'!D34/(Q28+R28+S28)*I28,0)+'M&amp;E'!E34+IFERROR('M&amp;E'!E34/R28*S28,0)+IFERROR(('M&amp;E'!E34+'M&amp;E'!E34/R28*S28)/(Q28+R28+S28)*I28,0))*Rates!$C$22)</f>
         <v/>
       </c>
       <c r="L28" s="161">
@@ -12316,7 +12324,7 @@
         <v/>
       </c>
       <c r="I29" s="155">
-        <f>IF(H29="","",Q29*Rates!$B$8)</f>
+        <f>IF(H29="","",(Q29+R29+S29)*Rates!$B$8)</f>
         <v/>
       </c>
       <c r="J29" s="154">
@@ -12324,7 +12332,7 @@
         <v/>
       </c>
       <c r="K29" s="155">
-        <f>IF(H29="","",(Labor!F37+IFERROR(Labor!F37/Q29*I29,0)+Labor!G37)*Rates!$C$19+(Travel!D35+IFERROR(Travel!D35/Q29*I29,0)+Travel!E35+IFERROR(Travel!E35/R29*S29,0))*Rates!$C$20+(ODCs!D35+IFERROR(ODCs!D35/Q29*I29,0)+ODCs!E35+IFERROR(ODCs!E35/R29*S29,0))*Rates!$C$21+('M&amp;E'!D35+IFERROR('M&amp;E'!D35/Q29*I29,0)+'M&amp;E'!E35+IFERROR('M&amp;E'!E35/R29*S29,0))*Rates!$C$22)</f>
+        <f>IF(H29="","",(Labor!F37+IFERROR(Labor!F37/(Q29+R29+S29)*I29,0)+Labor!G37)*Rates!$C$19+(Travel!D35+IFERROR(Travel!D35/(Q29+R29+S29)*I29,0)+Travel!E35+IFERROR(Travel!E35/R29*S29,0)+IFERROR((Travel!E35+Travel!E35/R29*S29)/(Q29+R29+S29)*I29,0))*Rates!$C$20+(ODCs!D35+IFERROR(ODCs!D35/(Q29+R29+S29)*I29,0)+ODCs!E35+IFERROR(ODCs!E35/R29*S29,0)+IFERROR((ODCs!E35+ODCs!E35/R29*S29)/(Q29+R29+S29)*I29,0))*Rates!$C$21+('M&amp;E'!D35+IFERROR('M&amp;E'!D35/(Q29+R29+S29)*I29,0)+'M&amp;E'!E35+IFERROR('M&amp;E'!E35/R29*S29,0)+IFERROR(('M&amp;E'!E35+'M&amp;E'!E35/R29*S29)/(Q29+R29+S29)*I29,0))*Rates!$C$22)</f>
         <v/>
       </c>
       <c r="L29" s="154">
@@ -12393,7 +12401,7 @@
         <v/>
       </c>
       <c r="I30" s="162">
-        <f>IF(H30="","",Q30*Rates!$B$8)</f>
+        <f>IF(H30="","",(Q30+R30+S30)*Rates!$B$8)</f>
         <v/>
       </c>
       <c r="J30" s="161">
@@ -12401,7 +12409,7 @@
         <v/>
       </c>
       <c r="K30" s="162">
-        <f>IF(H30="","",(Labor!F38+IFERROR(Labor!F38/Q30*I30,0)+Labor!G38)*Rates!$C$19+(Travel!D36+IFERROR(Travel!D36/Q30*I30,0)+Travel!E36+IFERROR(Travel!E36/R30*S30,0))*Rates!$C$20+(ODCs!D36+IFERROR(ODCs!D36/Q30*I30,0)+ODCs!E36+IFERROR(ODCs!E36/R30*S30,0))*Rates!$C$21+('M&amp;E'!D36+IFERROR('M&amp;E'!D36/Q30*I30,0)+'M&amp;E'!E36+IFERROR('M&amp;E'!E36/R30*S30,0))*Rates!$C$22)</f>
+        <f>IF(H30="","",(Labor!F38+IFERROR(Labor!F38/(Q30+R30+S30)*I30,0)+Labor!G38)*Rates!$C$19+(Travel!D36+IFERROR(Travel!D36/(Q30+R30+S30)*I30,0)+Travel!E36+IFERROR(Travel!E36/R30*S30,0)+IFERROR((Travel!E36+Travel!E36/R30*S30)/(Q30+R30+S30)*I30,0))*Rates!$C$20+(ODCs!D36+IFERROR(ODCs!D36/(Q30+R30+S30)*I30,0)+ODCs!E36+IFERROR(ODCs!E36/R30*S30,0)+IFERROR((ODCs!E36+ODCs!E36/R30*S30)/(Q30+R30+S30)*I30,0))*Rates!$C$21+('M&amp;E'!D36+IFERROR('M&amp;E'!D36/(Q30+R30+S30)*I30,0)+'M&amp;E'!E36+IFERROR('M&amp;E'!E36/R30*S30,0)+IFERROR(('M&amp;E'!E36+'M&amp;E'!E36/R30*S30)/(Q30+R30+S30)*I30,0))*Rates!$C$22)</f>
         <v/>
       </c>
       <c r="L30" s="161">
@@ -12470,7 +12478,7 @@
         <v/>
       </c>
       <c r="I31" s="155">
-        <f>IF(H31="","",Q31*Rates!$B$8)</f>
+        <f>IF(H31="","",(Q31+R31+S31)*Rates!$B$8)</f>
         <v/>
       </c>
       <c r="J31" s="154">
@@ -12478,7 +12486,7 @@
         <v/>
       </c>
       <c r="K31" s="155">
-        <f>IF(H31="","",(Labor!F39+IFERROR(Labor!F39/Q31*I31,0)+Labor!G39)*Rates!$C$19+(Travel!D37+IFERROR(Travel!D37/Q31*I31,0)+Travel!E37+IFERROR(Travel!E37/R31*S31,0))*Rates!$C$20+(ODCs!D37+IFERROR(ODCs!D37/Q31*I31,0)+ODCs!E37+IFERROR(ODCs!E37/R31*S31,0))*Rates!$C$21+('M&amp;E'!D37+IFERROR('M&amp;E'!D37/Q31*I31,0)+'M&amp;E'!E37+IFERROR('M&amp;E'!E37/R31*S31,0))*Rates!$C$22)</f>
+        <f>IF(H31="","",(Labor!F39+IFERROR(Labor!F39/(Q31+R31+S31)*I31,0)+Labor!G39)*Rates!$C$19+(Travel!D37+IFERROR(Travel!D37/(Q31+R31+S31)*I31,0)+Travel!E37+IFERROR(Travel!E37/R31*S31,0)+IFERROR((Travel!E37+Travel!E37/R31*S31)/(Q31+R31+S31)*I31,0))*Rates!$C$20+(ODCs!D37+IFERROR(ODCs!D37/(Q31+R31+S31)*I31,0)+ODCs!E37+IFERROR(ODCs!E37/R31*S31,0)+IFERROR((ODCs!E37+ODCs!E37/R31*S31)/(Q31+R31+S31)*I31,0))*Rates!$C$21+('M&amp;E'!D37+IFERROR('M&amp;E'!D37/(Q31+R31+S31)*I31,0)+'M&amp;E'!E37+IFERROR('M&amp;E'!E37/R31*S31,0)+IFERROR(('M&amp;E'!E37+'M&amp;E'!E37/R31*S31)/(Q31+R31+S31)*I31,0))*Rates!$C$22)</f>
         <v/>
       </c>
       <c r="L31" s="154">
@@ -12547,7 +12555,7 @@
         <v/>
       </c>
       <c r="I32" s="162">
-        <f>IF(H32="","",Q32*Rates!$B$8)</f>
+        <f>IF(H32="","",(Q32+R32+S32)*Rates!$B$8)</f>
         <v/>
       </c>
       <c r="J32" s="161">
@@ -12555,7 +12563,7 @@
         <v/>
       </c>
       <c r="K32" s="162">
-        <f>IF(H32="","",(Labor!F40+IFERROR(Labor!F40/Q32*I32,0)+Labor!G40)*Rates!$C$19+(Travel!D38+IFERROR(Travel!D38/Q32*I32,0)+Travel!E38+IFERROR(Travel!E38/R32*S32,0))*Rates!$C$20+(ODCs!D38+IFERROR(ODCs!D38/Q32*I32,0)+ODCs!E38+IFERROR(ODCs!E38/R32*S32,0))*Rates!$C$21+('M&amp;E'!D38+IFERROR('M&amp;E'!D38/Q32*I32,0)+'M&amp;E'!E38+IFERROR('M&amp;E'!E38/R32*S32,0))*Rates!$C$22)</f>
+        <f>IF(H32="","",(Labor!F40+IFERROR(Labor!F40/(Q32+R32+S32)*I32,0)+Labor!G40)*Rates!$C$19+(Travel!D38+IFERROR(Travel!D38/(Q32+R32+S32)*I32,0)+Travel!E38+IFERROR(Travel!E38/R32*S32,0)+IFERROR((Travel!E38+Travel!E38/R32*S32)/(Q32+R32+S32)*I32,0))*Rates!$C$20+(ODCs!D38+IFERROR(ODCs!D38/(Q32+R32+S32)*I32,0)+ODCs!E38+IFERROR(ODCs!E38/R32*S32,0)+IFERROR((ODCs!E38+ODCs!E38/R32*S32)/(Q32+R32+S32)*I32,0))*Rates!$C$21+('M&amp;E'!D38+IFERROR('M&amp;E'!D38/(Q32+R32+S32)*I32,0)+'M&amp;E'!E38+IFERROR('M&amp;E'!E38/R32*S32,0)+IFERROR(('M&amp;E'!E38+'M&amp;E'!E38/R32*S32)/(Q32+R32+S32)*I32,0))*Rates!$C$22)</f>
         <v/>
       </c>
       <c r="L32" s="161">
@@ -12591,7 +12599,6 @@
         <v/>
       </c>
     </row>
-    <row r="33"/>
     <row r="34" ht="15" customHeight="1" s="109">
       <c r="A34" s="120">
         <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
@@ -12667,7 +12674,6 @@
       </c>
       <c r="P1" s="142" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3" ht="28" customHeight="1" s="109">
       <c r="A3" s="165" t="inlineStr">
         <is>
@@ -12805,7 +12811,7 @@
         <f>IF(A5="","",IF(L5="Prime",H5*(1+Rates!$B$6)*(1+Rates!$B$7)*(1+Rates!$B$8),H5))</f>
         <v/>
       </c>
-      <c r="N5" s="173">
+      <c r="N5" s="230">
         <f>IF(A5="","",IF(H5="","",IFERROR(M5/H5,"")))</f>
         <v/>
       </c>
@@ -12859,7 +12865,7 @@
         <f>IF(A6="","",IF(L6="Prime",H6*(1+Rates!$B$6)*(1+Rates!$B$7)*(1+Rates!$B$8),H6))</f>
         <v/>
       </c>
-      <c r="N6" s="183">
+      <c r="N6" s="231">
         <f>IF(A6="","",IF(H6="","",IFERROR(M6/H6,"")))</f>
         <v/>
       </c>
@@ -12913,7 +12919,7 @@
         <f>IF(A7="","",IF(L7="Prime",H7*(1+Rates!$B$6)*(1+Rates!$B$7)*(1+Rates!$B$8),H7))</f>
         <v/>
       </c>
-      <c r="N7" s="173">
+      <c r="N7" s="230">
         <f>IF(A7="","",IF(H7="","",IFERROR(M7/H7,"")))</f>
         <v/>
       </c>
@@ -12945,7 +12951,7 @@
         <f>IF(A8="","",IF(L8="Prime",H8*(1+Rates!$B$6)*(1+Rates!$B$7)*(1+Rates!$B$8),H8))</f>
         <v/>
       </c>
-      <c r="N8" s="183">
+      <c r="N8" s="231">
         <f>IF(A8="","",IF(H8="","",IFERROR(M8/H8,"")))</f>
         <v/>
       </c>
@@ -12977,7 +12983,7 @@
         <f>IF(A9="","",IF(L9="Prime",H9*(1+Rates!$B$6)*(1+Rates!$B$7)*(1+Rates!$B$8),H9))</f>
         <v/>
       </c>
-      <c r="N9" s="173">
+      <c r="N9" s="230">
         <f>IF(A9="","",IF(H9="","",IFERROR(M9/H9,"")))</f>
         <v/>
       </c>
@@ -13009,7 +13015,7 @@
         <f>IF(A10="","",IF(L10="Prime",H10*(1+Rates!$B$6)*(1+Rates!$B$7)*(1+Rates!$B$8),H10))</f>
         <v/>
       </c>
-      <c r="N10" s="183">
+      <c r="N10" s="231">
         <f>IF(A10="","",IF(H10="","",IFERROR(M10/H10,"")))</f>
         <v/>
       </c>
@@ -13041,7 +13047,7 @@
         <f>IF(A11="","",IF(L11="Prime",H11*(1+Rates!$B$6)*(1+Rates!$B$7)*(1+Rates!$B$8),H11))</f>
         <v/>
       </c>
-      <c r="N11" s="173">
+      <c r="N11" s="230">
         <f>IF(A11="","",IF(H11="","",IFERROR(M11/H11,"")))</f>
         <v/>
       </c>
@@ -13073,7 +13079,7 @@
         <f>IF(A12="","",IF(L12="Prime",H12*(1+Rates!$B$6)*(1+Rates!$B$7)*(1+Rates!$B$8),H12))</f>
         <v/>
       </c>
-      <c r="N12" s="183">
+      <c r="N12" s="231">
         <f>IF(A12="","",IF(H12="","",IFERROR(M12/H12,"")))</f>
         <v/>
       </c>
@@ -13105,7 +13111,7 @@
         <f>IF(A13="","",IF(L13="Prime",H13*(1+Rates!$B$6)*(1+Rates!$B$7)*(1+Rates!$B$8),H13))</f>
         <v/>
       </c>
-      <c r="N13" s="173">
+      <c r="N13" s="230">
         <f>IF(A13="","",IF(H13="","",IFERROR(M13/H13,"")))</f>
         <v/>
       </c>
@@ -13137,7 +13143,7 @@
         <f>IF(A14="","",IF(L14="Prime",H14*(1+Rates!$B$6)*(1+Rates!$B$7)*(1+Rates!$B$8),H14))</f>
         <v/>
       </c>
-      <c r="N14" s="183">
+      <c r="N14" s="231">
         <f>IF(A14="","",IF(H14="","",IFERROR(M14/H14,"")))</f>
         <v/>
       </c>
@@ -13169,7 +13175,7 @@
         <f>IF(A15="","",IF(L15="Prime",H15*(1+Rates!$B$6)*(1+Rates!$B$7)*(1+Rates!$B$8),H15))</f>
         <v/>
       </c>
-      <c r="N15" s="173">
+      <c r="N15" s="230">
         <f>IF(A15="","",IF(H15="","",IFERROR(M15/H15,"")))</f>
         <v/>
       </c>
@@ -13201,7 +13207,7 @@
         <f>IF(A16="","",IF(L16="Prime",H16*(1+Rates!$B$6)*(1+Rates!$B$7)*(1+Rates!$B$8),H16))</f>
         <v/>
       </c>
-      <c r="N16" s="183">
+      <c r="N16" s="231">
         <f>IF(A16="","",IF(H16="","",IFERROR(M16/H16,"")))</f>
         <v/>
       </c>
@@ -13233,7 +13239,7 @@
         <f>IF(A17="","",IF(L17="Prime",H17*(1+Rates!$B$6)*(1+Rates!$B$7)*(1+Rates!$B$8),H17))</f>
         <v/>
       </c>
-      <c r="N17" s="173">
+      <c r="N17" s="230">
         <f>IF(A17="","",IF(H17="","",IFERROR(M17/H17,"")))</f>
         <v/>
       </c>
@@ -13265,7 +13271,7 @@
         <f>IF(A18="","",IF(L18="Prime",H18*(1+Rates!$B$6)*(1+Rates!$B$7)*(1+Rates!$B$8),H18))</f>
         <v/>
       </c>
-      <c r="N18" s="183">
+      <c r="N18" s="231">
         <f>IF(A18="","",IF(H18="","",IFERROR(M18/H18,"")))</f>
         <v/>
       </c>
@@ -13297,7 +13303,7 @@
         <f>IF(A19="","",IF(L19="Prime",H19*(1+Rates!$B$6)*(1+Rates!$B$7)*(1+Rates!$B$8),H19))</f>
         <v/>
       </c>
-      <c r="N19" s="173">
+      <c r="N19" s="230">
         <f>IF(A19="","",IF(H19="","",IFERROR(M19/H19,"")))</f>
         <v/>
       </c>
@@ -13391,7 +13397,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="28" customHeight="1" s="109">
       <c r="A3" s="114" t="inlineStr">
         <is>
@@ -13421,73 +13426,73 @@
           <t>Jan</t>
         </is>
       </c>
-      <c r="E4" s="187" t="n"/>
+      <c r="E4" s="232" t="n"/>
       <c r="F4" s="186" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="G4" s="187" t="n"/>
+      <c r="G4" s="232" t="n"/>
       <c r="H4" s="186" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="I4" s="187" t="n"/>
+      <c r="I4" s="232" t="n"/>
       <c r="J4" s="186" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="K4" s="187" t="n"/>
+      <c r="K4" s="232" t="n"/>
       <c r="L4" s="186" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="M4" s="187" t="n"/>
+      <c r="M4" s="232" t="n"/>
       <c r="N4" s="186" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="O4" s="187" t="n"/>
+      <c r="O4" s="232" t="n"/>
       <c r="P4" s="186" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
-      <c r="Q4" s="187" t="n"/>
+      <c r="Q4" s="232" t="n"/>
       <c r="R4" s="186" t="inlineStr">
         <is>
           <t>Aug</t>
         </is>
       </c>
-      <c r="S4" s="187" t="n"/>
+      <c r="S4" s="232" t="n"/>
       <c r="T4" s="186" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="U4" s="187" t="n"/>
+      <c r="U4" s="232" t="n"/>
       <c r="V4" s="186" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="W4" s="187" t="n"/>
+      <c r="W4" s="232" t="n"/>
       <c r="X4" s="186" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
-      <c r="Y4" s="187" t="n"/>
+      <c r="Y4" s="232" t="n"/>
       <c r="Z4" s="186" t="inlineStr">
         <is>
           <t>Dec</t>
         </is>
       </c>
-      <c r="AA4" s="187" t="n"/>
+      <c r="AA4" s="232" t="n"/>
       <c r="AB4" s="126" t="inlineStr">
         <is>
           <t>Yearly
@@ -13502,9 +13507,9 @@
       </c>
     </row>
     <row r="5" ht="28" customHeight="1" s="109">
-      <c r="A5" s="188" t="n"/>
-      <c r="B5" s="188" t="n"/>
-      <c r="C5" s="188" t="n"/>
+      <c r="A5" s="233" t="n"/>
+      <c r="B5" s="233" t="n"/>
+      <c r="C5" s="233" t="n"/>
       <c r="D5" s="137" t="inlineStr">
         <is>
           <t>Planned
@@ -13649,8 +13654,8 @@
 Hrs</t>
         </is>
       </c>
-      <c r="AB5" s="188" t="n"/>
-      <c r="AC5" s="188" t="n"/>
+      <c r="AB5" s="233" t="n"/>
+      <c r="AC5" s="233" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1" s="109">
       <c r="A6" s="128" t="n">
@@ -14235,7 +14240,6 @@
         <v/>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="117">
         <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
@@ -14246,10 +14250,10 @@
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="B0B1"/>
   <mergeCells count="18">
     <mergeCell ref="F4:G4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="X4:Y4"/>
     <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="X4:Y4"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="A3:AA3"/>
     <mergeCell ref="L4:M4"/>
@@ -14352,7 +14356,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="109">
       <c r="A3" s="117" t="inlineStr">
         <is>
@@ -14406,97 +14409,97 @@
           <t>Jan</t>
         </is>
       </c>
-      <c r="I4" s="194" t="n"/>
-      <c r="J4" s="194" t="n"/>
-      <c r="K4" s="187" t="n"/>
+      <c r="I4" s="234" t="n"/>
+      <c r="J4" s="234" t="n"/>
+      <c r="K4" s="232" t="n"/>
       <c r="L4" s="186" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="M4" s="194" t="n"/>
-      <c r="N4" s="194" t="n"/>
-      <c r="O4" s="187" t="n"/>
+      <c r="M4" s="234" t="n"/>
+      <c r="N4" s="234" t="n"/>
+      <c r="O4" s="232" t="n"/>
       <c r="P4" s="186" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="Q4" s="194" t="n"/>
-      <c r="R4" s="194" t="n"/>
-      <c r="S4" s="187" t="n"/>
+      <c r="Q4" s="234" t="n"/>
+      <c r="R4" s="234" t="n"/>
+      <c r="S4" s="232" t="n"/>
       <c r="T4" s="186" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="U4" s="194" t="n"/>
-      <c r="V4" s="194" t="n"/>
-      <c r="W4" s="187" t="n"/>
+      <c r="U4" s="234" t="n"/>
+      <c r="V4" s="234" t="n"/>
+      <c r="W4" s="232" t="n"/>
       <c r="X4" s="186" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="Y4" s="194" t="n"/>
-      <c r="Z4" s="194" t="n"/>
-      <c r="AA4" s="187" t="n"/>
+      <c r="Y4" s="234" t="n"/>
+      <c r="Z4" s="234" t="n"/>
+      <c r="AA4" s="232" t="n"/>
       <c r="AB4" s="186" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="AC4" s="194" t="n"/>
-      <c r="AD4" s="194" t="n"/>
-      <c r="AE4" s="187" t="n"/>
+      <c r="AC4" s="234" t="n"/>
+      <c r="AD4" s="234" t="n"/>
+      <c r="AE4" s="232" t="n"/>
       <c r="AF4" s="186" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
-      <c r="AG4" s="194" t="n"/>
-      <c r="AH4" s="194" t="n"/>
-      <c r="AI4" s="187" t="n"/>
+      <c r="AG4" s="234" t="n"/>
+      <c r="AH4" s="234" t="n"/>
+      <c r="AI4" s="232" t="n"/>
       <c r="AJ4" s="186" t="inlineStr">
         <is>
           <t>Aug</t>
         </is>
       </c>
-      <c r="AK4" s="194" t="n"/>
-      <c r="AL4" s="194" t="n"/>
-      <c r="AM4" s="187" t="n"/>
+      <c r="AK4" s="234" t="n"/>
+      <c r="AL4" s="234" t="n"/>
+      <c r="AM4" s="232" t="n"/>
       <c r="AN4" s="186" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="AO4" s="194" t="n"/>
-      <c r="AP4" s="194" t="n"/>
-      <c r="AQ4" s="187" t="n"/>
+      <c r="AO4" s="234" t="n"/>
+      <c r="AP4" s="234" t="n"/>
+      <c r="AQ4" s="232" t="n"/>
       <c r="AR4" s="186" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="AS4" s="194" t="n"/>
-      <c r="AT4" s="194" t="n"/>
-      <c r="AU4" s="187" t="n"/>
+      <c r="AS4" s="234" t="n"/>
+      <c r="AT4" s="234" t="n"/>
+      <c r="AU4" s="232" t="n"/>
       <c r="AV4" s="186" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
-      <c r="AW4" s="194" t="n"/>
-      <c r="AX4" s="194" t="n"/>
-      <c r="AY4" s="187" t="n"/>
+      <c r="AW4" s="234" t="n"/>
+      <c r="AX4" s="234" t="n"/>
+      <c r="AY4" s="232" t="n"/>
       <c r="AZ4" s="186" t="inlineStr">
         <is>
           <t>Dec</t>
         </is>
       </c>
-      <c r="BA4" s="194" t="n"/>
-      <c r="BB4" s="194" t="n"/>
-      <c r="BC4" s="187" t="n"/>
+      <c r="BA4" s="234" t="n"/>
+      <c r="BB4" s="234" t="n"/>
+      <c r="BC4" s="232" t="n"/>
       <c r="BD4" s="126" t="inlineStr">
         <is>
           <t>Yearly Max
@@ -14523,13 +14526,13 @@
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" s="109">
-      <c r="A5" s="188" t="n"/>
-      <c r="B5" s="188" t="n"/>
-      <c r="C5" s="188" t="n"/>
-      <c r="D5" s="188" t="n"/>
-      <c r="E5" s="188" t="n"/>
-      <c r="F5" s="188" t="n"/>
-      <c r="G5" s="188" t="n"/>
+      <c r="A5" s="233" t="n"/>
+      <c r="B5" s="233" t="n"/>
+      <c r="C5" s="233" t="n"/>
+      <c r="D5" s="233" t="n"/>
+      <c r="E5" s="233" t="n"/>
+      <c r="F5" s="233" t="n"/>
+      <c r="G5" s="233" t="n"/>
       <c r="H5" s="137" t="inlineStr">
         <is>
           <t>Max
@@ -14818,10 +14821,10 @@
 $</t>
         </is>
       </c>
-      <c r="BD5" s="188" t="n"/>
-      <c r="BE5" s="188" t="n"/>
-      <c r="BF5" s="188" t="n"/>
-      <c r="BG5" s="188" t="n"/>
+      <c r="BD5" s="233" t="n"/>
+      <c r="BE5" s="233" t="n"/>
+      <c r="BF5" s="233" t="n"/>
+      <c r="BG5" s="233" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1" s="109">
       <c r="A6" s="128" t="n">
@@ -17829,7 +17832,6 @@
         <v/>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="123" t="inlineStr">
         <is>
@@ -18389,7 +18391,6 @@
         <v/>
       </c>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="A42" s="117" t="inlineStr">
         <is>
@@ -18397,7 +18398,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
     <row r="44">
       <c r="A44" s="117">
         <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
@@ -18420,9 +18420,9 @@
     <mergeCell ref="P4:S4"/>
     <mergeCell ref="H4:K4"/>
     <mergeCell ref="BD4:BD5"/>
+    <mergeCell ref="T4:W4"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="G4:G5"/>
-    <mergeCell ref="T4:W4"/>
     <mergeCell ref="AB4:AE4"/>
     <mergeCell ref="AN4:AQ4"/>
     <mergeCell ref="AF4:AI4"/>
@@ -18557,7 +18557,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="109">
       <c r="A3" s="123" t="inlineStr">
         <is>
@@ -18909,7 +18908,6 @@
         <v/>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="123" t="inlineStr">
         <is>
@@ -19203,7 +19201,6 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="117">
         <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>
@@ -19260,7 +19257,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="109">
       <c r="A3" s="123" t="inlineStr">
         <is>
@@ -19612,7 +19608,6 @@
         <v/>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="123" t="inlineStr">
         <is>
@@ -19906,7 +19901,6 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="117">
         <f>"Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com"&amp;IF(_License!$B$2="","","  ·  Licensed to: "&amp;_License!$B$2)</f>

</xml_diff>

<commit_message>
Add TOA definition to Excel tracker and clarify Dashboard label
Instructions tab now has a 'Key terms' section defining TOA (Total
Obligated Amount / Current Funding). The Dashboard's 'Current TOA'
label is now 'Current TOA (Current Funding)' so it's self-explanatory
without needing to check Instructions. Sheet protection and password
(unchanged) verified intact after the edit.
</commit_message>
<xml_diff>
--- a/client/public/examples/cost-and-burn-rate-tracker.xlsx
+++ b/client/public/examples/cost-and-burn-rate-tracker.xlsx
@@ -2799,10 +2799,23 @@
       <c r="A37" s="113" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1" s="109">
-      <c r="A38" s="113" t="n"/>
+      <c r="A38" s="115" t="inlineStr">
+        <is>
+          <t>Key terms</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="109">
-      <c r="A39" s="113" t="n"/>
+      <c r="A39" s="116" t="inlineStr">
+        <is>
+          <t>TOA</t>
+        </is>
+      </c>
+      <c r="B39" s="114" t="inlineStr">
+        <is>
+          <t>Total Obligated Amount (Current Funding). The total dollar amount funded on this contract or task order right now. It comes from the CONTRACT TOTAL row on the Projects tab, and the whole Dashboard (burn rate, % spent, months to exhaustion) is calculated against it.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="109">
       <c r="A40" s="113" t="n"/>
@@ -11467,7 +11480,7 @@
     <row r="8" ht="15" customHeight="1" s="109">
       <c r="A8" s="118" t="inlineStr">
         <is>
-          <t>Current TOA (from Projects tab)</t>
+          <t>Current TOA (Current Funding)</t>
         </is>
       </c>
       <c r="C8" s="146">

</xml_diff>